<commit_message>
feat: save updated video/photo titles and enable uploading both photos and videos in multimedia view
</commit_message>
<xml_diff>
--- a/Base_de_Datos_Giants.xlsx
+++ b/Base_de_Datos_Giants.xlsx
@@ -2374,7 +2374,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Nuevo Fichaje Oficial: Presentación con la equipación rosinegra</t>
+          <t>NUEVO FICHAJE: J. Epstein, dicen q es buen ojeador de filiales.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Nuevo Fichaje Oficial: Incorporación de garantía para la temporada</t>
+          <t>NUEVO FICHAJE: RHLM</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -2430,7 +2430,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Javier Chimeno #12 listo para saltar al terreno de juego</t>
+          <t>Javi poniéndose guantes, no sé pa q. No es portero.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Reunión táctica con el colegiado previo al choque</t>
+          <t>Amañando el partido ofreciéndole 2.500.000 millones de Bolívares (2€).</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Rubén Montes #10 conectando un potente disparo de zurda</t>
+          <t>Rubo dándole a la bola. Fútbol vaya.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Remate cruzado en zona de peligro del rival</t>
+          <t>No fue gol, tranquis.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Actualizacion de Temporada, modal de partidos, actas, base de datos de estadios y ajustes de interfaz para Poligono Giants
</commit_message>
<xml_diff>
--- a/Base_de_Datos_Giants.xlsx
+++ b/Base_de_Datos_Giants.xlsx
@@ -631,13 +631,13 @@
         <v>25</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>0</v>
@@ -652,7 +652,7 @@
         <v>0</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O3" s="2" t="n">
         <v>1</v>
@@ -1568,7 +1568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1641,7 +1641,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>next</t>
+          <t>past</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T20:30</t>
+          <t>2026-09-05T18:00</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1669,10 +1669,14 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
+      <c r="H2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="J2" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -1681,7 +1685,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>future</t>
+          <t>past</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1696,7 +1700,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T20:30</t>
+          <t>2026-09-12T19:30</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1709,10 +1713,14 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
+      <c r="H3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="J3" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1721,7 +1729,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>future</t>
+          <t>past</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1736,7 +1744,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T20:30</t>
+          <t>2026-09-19T17:00</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1749,8 +1757,12 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
+      <c r="H4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="J4" s="2" t="b">
         <v>0</v>
       </c>
@@ -1761,7 +1773,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>future</t>
+          <t>past</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1776,7 +1788,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T20:30</t>
+          <t>2026-09-26T18:00</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1789,10 +1801,14 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="2" t="n"/>
+      <c r="H5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="J5" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1801,7 +1817,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>future</t>
+          <t>past</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1816,7 +1832,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T20:30</t>
+          <t>2026-10-03T19:00</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1829,8 +1845,12 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
+      <c r="H6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="J6" s="2" t="b">
         <v>0</v>
       </c>
@@ -1841,7 +1861,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>future</t>
+          <t>past</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1856,7 +1876,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-11-05T20:30</t>
+          <t>2026-10-10T20:30</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1869,10 +1889,14 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
+      <c r="H7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="J7" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -1881,7 +1905,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>future</t>
+          <t>next</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1896,7 +1920,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-11-12T20:30</t>
+          <t>2026-10-18T19:30</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1909,11 +1933,9 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1936,7 +1958,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2026-11-19T20:30</t>
+          <t>2026-10-25T18:00</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1949,11 +1971,9 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
-      <c r="J9" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1976,7 +1996,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-11-26T20:30</t>
+          <t>2026-11-01T17:00</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1989,11 +2009,9 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -2016,7 +2034,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2026-12-03T20:30</t>
+          <t>2026-11-08T19:00</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -2029,11 +2047,9 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -2056,7 +2072,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-12-10T20:30</t>
+          <t>2026-11-15T18:30</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -2069,11 +2085,9 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -2096,7 +2110,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-12-17T20:30</t>
+          <t>2026-11-22T20:00</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -2109,11 +2123,47 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
-      <c r="J13" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>113</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>future</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Liga F7 Gijón - Jornada 13</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Rayo La Arena</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-29T17:30</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Campo Municipal La Camocha (Gijón)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2277,7 +2327,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAABAAAAAYACAIAAABn4K39AAEOkmNhQlgAAQ6SanVtYgAAAB5qdW1kYzJwYQARABCAAACqADibcQNjMnBhAAAANvpqdW1iAAAAR2p1bWRjMm1hABEAEIAAAKoAOJtxA3VybjpjMnBhOmRiMGE3MzlmLTNjMjYtNGQ3NC1iODZlLTVkNjE0MzM1NWExNgAAAAHBanVtYgAAAClqdW1kYzJhcwARABCAAACqADibcQNjMnBhLmFzc2VydGlvbnMAAAAA5Wp1bWIAAAApanVtZGNib3IAEQAQgAAAqgA4m3EDYzJwYS5hY3Rpb25zLnYyAAAAALRjYm9yoWdhY3Rpb25zgqNmYWN0aW9ubGMycGEuY3JlYXRlZG1zb2Z0d2FyZUFnZW50v2RuYW1lZkdQVC00b/9xZGlnaXRhbFNvdXJjZVR5cGV4Rmh0dHA6Ly9jdi5pcHRjLm9yZy9uZXdzY29kZXMvZGlnaXRhbHNvdXJjZXR5cGUvdHJhaW5lZEFsZ29yaXRobWljTWVkaWGhZmFjdGlvbm5jMnBhLmNvbnZlcnRlZAAAAKtqdW1iAAAAKGp1bWRjYm9yABEAEIAAAKoAOJtxA2MycGEuaGFzaC5kYXRhAAAAAHtjYm9ypWpleGNsdXNpb25zgaJlc3RhcnQYIWZsZW5ndGgZNyxkbmFtZW5qdW1iZiBtYW5pZmVzdGNhbGdmc2hhMjU2ZGhhc2hYIN0AGGD8R+jIO9op915Jl8vl3mHtLAjGrCa2On11sqCPY3BhZEgAAAAAAAAAAAAAAe1qdW1iAAAAJ2p1bWRjMmNsABEAEIAAAKoAOJtxA2MycGEuY2xhaW0udjIAAAABvmNib3Kmamluc3RhbmNlSUR4LHhtcDppaWQ6MTRkYmZlZTQtMzAxMC00NDNjLWE2NjMtODQ1YjkwYmJiZjk2dGNsYWltX2dlbmVyYXRvcl9pbmZvv2RuYW1lZ0NoYXRHUFR3b3JnLmNvbnRlbnRhdXRoLmMycGFfcnNlMC4wLjD/aXNpZ25hdHVyZXhNc2VsZiNqdW1iZj0vYzJwYS91cm46YzJwYTpkYjBhNzM5Zi0zYzI2LTRkNzQtYjg2ZS01ZDYxNDMzNTVhMTYvYzJwYS5zaWduYXR1cmVyY3JlYXRlZF9hc3NlcnRpb25zgqJjdXJseCpzZWxmI2p1bWJmPWMycGEuYXNzZXJ0aW9ucy9jMnBhLmFjdGlvbnMudjJkaGFzaFggj06jKi2a0YnaYj1JQTJA/fXaKbmaViQasY2WYTITPLWiY3VybHgpc2VsZiNqdW1iZj1jMnBhLmFzc2VydGlvbnMvYzJwYS5oYXNoLmRhdGFkaGFzaFgg+3M53OYYcLScqzfHzBqEic+qh6/E0/rAp5JIjOSKA5JoZGM6dGl0bGVpaW1hZ2UucG5nY2FsZ2ZzaGEyNTYAADL9anVtYgAAAChqdW1kYzJjcwARABCAAACqADibcQNjMnBhLnNpZ25hdHVyZQAAADLNY2JvctKEWQfBogEmGCGCWQM3MIIDMzCCAhugAwIBAgIUbq4oo+7FuOQqNvod5kEVrmIWGzswDQYJKoZIhvcNAQEMBQAwSjEaMBgGA1UEAwwRV2ViQ2xhaW1TaWduaW5nQ0ExDTALBgNVBAsMBExlbnMxEDAOBgNVBAoMB1RydWVwaWMxCzAJBgNVBAYTAlVTMB4XDTI1MDExMzIwMzY0NloXDTI2MDExMzIwMzY0NVowVjELMAkGA1UEBhMCVVMxDzANBgNVBAoMBk9wZW5BSTEQMA4GA1UECwwHQ2hhdEdQVDEkMCIGA1UEAwwbVHJ1ZXBpYyBMZW5zIENMSSBpbiBDaGF0R1BUMFkwEwYHKoZIzj0CAQYIKoZIzj0DAQcDQgAEVh14xypQD33uBMgU9aukdnuL7dOjIz3VpkIz2UwpCUIxMAhLpTWV6JHjLvDamqOsAQruAtmJXwzVLbsuFpo36KOBzzCBzDAMBgNVHRMBAf8EAjAAMB8GA1UdIwQYMBaAFFofa2bTlOewQYN9nAx7XcVzS0uzME0GCCsGAQUFBwEBBEEwPzA9BggrBgEFBQcwAYYxaHR0cDovL3ZhLnRydWVwaWMuY29tL2VqYmNhL3B1YmxpY3dlYi9zdGF0dXMvb2NzcDAdBgNVHSUEFjAUBggrBgEFBQcDBAYIKwYBBQUHAyQwHQYDVR0OBBYEFMpeEy4sGzWibWJFTTNDBWLsk/gqMA4GA1UdDwEB/wQEAwIHgDANBgkqhkiG9w0BAQwFAAOCAQEAeWg+ez3jguHZXbm4bruh1xJE0JcUKfUHUy3T9/qn0/I94RHpAuJHGtOR82heKf3qzXyKXu3rRh/w5kFKudwDaaqvxVpD2UXLAK+N9Nxqr02LLYybAJ8z04PrvS3pWKY3F5PvoV5nxA9DpHbJVSBJBt+xGo2atxcCGn0DenxkH7pRhqD+nYFivtypiEnuwNH8JrUbjRPJa07iMEfe9I7UEfsXPCisg0hxTFlMZPJkxqzqA6OvS71q+KQqg2qTzuZljF2JIQs1lWyROHBwZS2lZbruxqDTLu+uva49Rgq9XwQV9CeaEO+aRKW2QQgp/S+IQJK8Lv0U1GN3qWhnDxgBylkEfjCCBHowggJioAMCAQICFGn8kMTMiVCCOh6oX9KC/yjV/ZOQMA0GCSqGSIb3DQEBDAUAMD8xDzANBgNVBAMMBlJvb3RDQTENMAsGA1UECwwETGVuczEQMA4GA1UECgwHVHJ1ZXBpYzELMAkGA1UEBhMCVVMwHhcNMjExMjA5MjAzOTQ2WhcNMjYxMjA4MjAzOTQ1WjBKMRowGAYDVQQDDBFXZWJDbGFpbVNpZ25pbmdDQTENMAsGA1UECwwETGVuczEQMA4GA1UECgwHVHJ1ZXBpYzELMAkGA1UEBhMCVVMwggEiMA0GCSqGSIb3DQEBAQUAA4IBDwAwggEKAoIBAQDBFhLDp1DBmMzOa/iOpPHFavpylojYBTP7iuyC8mWA50GcmsThYBXHBOgoa/XH2t4KiiL6xaej9goo/gdiOwrLCXlleQ5YmpQ8li8vYtUWWMyKqJfKSJACWesINuevL6U9+3+T73exvuh6OPgUHkQXUGjh+WepF0n1v03K+/a8gaGfZEjhWAh6XKt6QfuGhjoBoe6mct4got3CqFE1nYyXq3J0MvkTm5v6u1n91NhXTMit76FxH4VsH+fYHfC9KuQ0Zoi+mROwfbHfYW3Nvm7W89/oMxdTKv8DdZajmtvnFiqRHRjHS7YDEVTW85nGcYuTvnBSuRLlxoV9aBjBArJvAgMBAAGjYzBhMA8GA1UdEwEB/wQFMAMBAf8wHwYDVR0jBBgwFoAUWLrxqfIN50UGCrApp1qXMOonPQswHQYDVR0OBBYEFFofa2bTlOewQYN9nAx7XcVzS0uzMA4GA1UdDwEB/wQEAwIBhjANBgkqhkiG9w0BAQwFAAOCAgEAdTiGehcRQvBXfAawu3fdO42FymnF5EFaM4wheoZxf0Xti3xT0KrnMbhzP3dTYaBhn6ZOherz8Mg924znkFcVsF98kTZjk6loVulFx087JxSKnJJrAV2CKwdHy9EEVj+r1EMbLjQW6tJT0KINCuWNlxdEDhm7/9lhhgbCe01bWn8OcVlfONX/duGO350pM0Bi6iWj2iYVVcnlfFAwoT9KobjdkXpLfAuoJMjUK+KV05YCzKoC1Q+1xsKy98JAACCz4ss+0dbJya1Ci2FdrL5D5/erUAehjruC7ZNvQepsqJyMBxz0H5bEJeFdvMcNpawC7bmTrWkq+OwrNjhrP8J+iIltHBBQnnfLJqFHtOQb2ThKvkuDtj0ist0EP1KFom+0EImvO16l6Dl0/AYubyPFJfuSM6sXs6ZgEBFz370+i7Ug7TkuqHcETkLEvBa2uC1BIlScnh5MwFyaEn9V3YSinECYaIrlaf/ksrubk7n/Skt1XXMs7kTKZsFhJ3HsUKkj0yFRNoGNq1aPpngJG91V8nRTM/kV5zCnSRNMuagjsrGq/qXU38rUxTe3PInYPrOuzklvTGzJSHvr81GO34zX03wA0GmYMqWUMZaYwSbnIQkdGue3WnA24NUpEp+kwm+KxW3juwkp/4KKeFWuYYkqu3vpn/1Q/55cRGK23YIn6dGhY3BhZFkqtAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAPZYQF79EBopRsDfAEl0DU8qL+x20yfEJj/9JiDANNnhQY69daT5v5I5LdePooG+05p6F5IbCgUmK2STZxc2okpLtvQAANdyanVtYgAAAEdqdW1kYzJtYQARABCAAACqADibcQN1cm46YzJwYTpjNGQ0NWY1Ni04ZDE3LTQxMDItOWU2Yi0xOWQ0ZjliMGYyZjAAAAChZ2p1bWIAAAApanVtZGMyYXMAEQAQgAAAqgA4m3EDYzJwYS5hc3NlcnRpb25zAAAAmddqdW1iAAAAS2p1bWRAywwyu4pInacLKtb0f0NpE2MycGEudGh1bWJuYWlsLmluZ3JlZGllbnQAAAAAGGMyc2hcQb0zUge9azgVV8EFyNLWAAAAFGJmZGIAaW1hZ2UvanBlZwAAAJlwYmlkYv/Y/+AAEEpGSUYAAQIAAAEAAQAA/8AAEQgB9AFNAwERAAIRAQMRAf/bAEMABgQFBgUEBgYFBgcHBggKEAoKCQkKFA4PDBAXFBgYFxQWFhodJR8aGyMcFhYgLCAjJicpKikZHy0wLSgwJSgpKP/bAEMBBwcHCggKEwoKEygaFhooKCgoKCgoKCgoKCgoKCgoKCgoKCgoKCgoKCgoKCgoKCgoKCgoKCgoKCgoKCgoKCgoKP/EAB8AAAEFAQEBAQEBAAAAAAAAAAABAgMEBQYHCAkKC//EALUQAAIBAwMCBAMFBQQEAAABfQECAwAEEQUSITFBBhNRYQcicRQygZGhCCNCscEVUtHwJDNicoIJChYXGBkaJSYnKCkqNDU2Nzg5OkNERUZHSElKU1RVVldYWVpjZGVmZ2hpanN0dXZ3eHl6g4SFhoeIiYqSk5SVlpeYmZqio6Slpqeoqaqys7S1tre4ubrCw8TFxsfIycrS09TV1tfY2drh4uPk5ebn6Onq8fLz9PX29/j5+v/EAB8BAAMBAQEBAQEBAQEAAAAAAAABAgMEBQYHCAkKC//EALURAAIBAgQEAwQHBQQEAAECdwABAgMRBAUhMQYSQVEHYXETIjKBCBRCkaGxwQkjM1LwFWJy0QoWJDThJfEXGBkaJicoKSo1Njc4OTpDREVGR0hJSlNUVVZXWFlaY2RlZmdoaWpzdHV2d3h5eoKDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usLDxMXGx8jJytLT1NXW19jZ2uLj5OXm5+jp6vLz9PX29/j5+v/aAAwDAQACEQMRAD8A+paACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgDnPF3jPRPClr52r3YVicLDEN8jH2Uc9utAHguu/tAa4mrrNY2Nta6eTtW3ueZGHXccYIz2pDK9x+0Lr0uEht9NikLbuMt8vpjP60AejeCfjpoOrkWuvo2j3wKpuky0MhPcOOg+vr1piPT9K1rS9W3/2XqNpeeX97yJVfb9cGgDQoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKAMjxP4k0rwxprX2tXa28AOBkZLH0AHJoC1zx/wAY/H60gEkPhmzNz8gIup8qoJ9F6nFTcrlPnPXfEepa1qjXV1cNNPIcmTjA5OAvsM00gMaWIIykhmYnknnJoENTAJWFQJOuVHI/GmBNaapf2Emd2AQRz3B4I/GgDc8KeL7rRNSjurKIWssZBR15x9eaQz2rSPjzqVvbxLqNrBdFukqnbkfSldj5UeiWXxq8LPpr3V9LLaOgH7p1yWPoMcU7ktWJJ/jV4NhlgV7ycpKoYSCE7VJ7H3ouFjpbTx54WuhF5WvafmQZVWmCk/gaLoLM6RWDKGUgqRkEd6YhaACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgCjrWrWGiWD3uq3UdtbJ1eQ4GfSgD4x+MXjf8A4SbxVdXVuZZbJG22yNkqAO+PU1O5exwbXLy22+VSfYDJosFypHcusjM4KKO3c1RJNNLNcoghJDZwQpA5pXsPc2bXw7epAJLq4jVTjPPT2rL2q2NlQdrtmfqRjgkaOKLz2Vtu7Pf/AArRaq7MmrOyGWkFxv8AMnt3WPHHbFLmQ+V7sdK6MFhV2EZJ2HupxVE+Q9NKuZw0ceWI5wSeaXMPkZGiyW0RhWaYMf4XA600xEME9x5vlSuSxzt3DofSmI+rP2cviBc63bnwzqQWSaxthJBcAkFowQNrA9xkc+lIGe4UxBQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFAEV1OltbTTynEcSF2PsBmgD4z+MvxHuvFmrzQxXWNGtmzFGvAJHBJPeo3L2PLbTfd3BaVtiuePpTbsJajD5slw0NohZRyzdce+fpQ3bcaTexJLBuuY4mb5y2M9R+FJvS40tbG8PDty8wMDCNAF5AwelZe1S0N/YNu50fmRQaYbFpleUclt3B/HFQr35jV2UeU4O6iuBds0O50yenQ+9dCkjjcXfQ15vtqaPtk+Ykg9c4rPTmNnzKJVsfJkQLcowkD8Y9x/wDWq3foZRS6nSXIc6ORbuI5lOA2ME4Hes09Tdr3TkRc3Lzu1yuZTgDJ4NbpnKx11Mr3CszBnbG73NCdwZ6D8F/EC6V8RNLkt2Mau6wSDH3lc7SP1B/Ck9B7o+16ogKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoA87+PfiCTQPhvqJtpHju7wC1iZFzjd97Oeny5pMaPiGe3e4ufKU9hn/aap2RVruxb1GOGxhjt7Zt90xw8h6D2FJX3G0loi/o0UEBWOBcvjLuxzn14rOd92b07bI6+18KQ+al0BHHKV6Fc7c+lc7qvY61QjuW7vSp2AjguVWM8MduDSU7blSpt6JlZvB+V+aUEH1zV+3ZH1a5G/hMsreW8YPbb8vPrTVYTw5VutGu7JuJJXUjDZGQT9M9KpTTIdKUSnNA4ViUjTIwOMc+opqRLh3INShnubLEUgYr94qefxqoySepE4NrQ5xY5YbeZx/r1IKk/WtuY5uXTUim3XCCdVHmockAYzx6UxGhok1xazw31m+xkZWVh1VgQf580mhpn3l4E1dtd8IaXqMrK0s8KmTaeN3Q01qS9Gb1MQUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFAHhv7VniQ6b4Ot9Lt54xJey4ljwGbYORxnIGcc0mNHy1YwsnmzYLtk7OetQy0iikU11ctJMNuOBTbBRuzp/DVm32yJXV9jPznjOOaxqPQ6aMbM9OLZAAAzXJY77kQ+9knJqrBctb3ZDjHvRygpEcXVi5Oe1KwyCfPmccrRyjuV5o4pl8qeNWA7EZxS1QNJ7mTNpVsC5hkeJmHTqtaKb6mLpLoYl/pTpbMGG/vuXvW0Z6nPOnoZtt5dkXcoN6nIDDPNbJ3OZpRF022M0Ny8ICbBvZMd8/wCBpt20JSvqj6D/AGYfEivb3+hz3W5g3nwRMfu/3gPxx+dOJMl1PfaogKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgD40/akuoNS+J6WttcJN5NuiyBTny2GSV9j0/OpZSONsLFmt9zDHGR/OsnI3jAkh0o4yqZxnA9wM1LkaKBsaLE9vN+/UebnruyQKym7m9ONtzpxKxXHGM1Bt1GqT2Yj2oQNGja4fCZ+lWlchuxfa3QIQoXpjNVyonmZSmhAzxWb0NU7mXdMFbPrUGtynKN3IpohkYkVRg9aoRB9lhu5AG6nuBWkG0zCpBNDtZ0+XSbdFjt1khdS7S7PmHSuh6o41ozltE1P+wvGFtfxNuijkEx5PTr2poiR94aTfQ6npdrfWriSC4jWRGHcEVZkW6ACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgD4n8X+HbU/GDWYYrkXENvI0s5Ts7HO3Pc561lN2RtTV2aklrEu4oo8vAUDHT2rA6rWKzW/lSAqo4zgenNSzSJIYwWDHjHQVBqAmbzAq8AdDQNEwId8g9T0JqhMuxvtjBAPHoapE7lyO6Lccg+56UXCwksvUHknp7VLLRnXaqeen+FSX0KwVVUg/Tg07E3KVxEQ+7ORVWJY/TiBdoWIAzVRRnNnb6b5d5C0NwMxlSjfStrnM0eJ+LPLh8Wz2m5RiYx7uwHSqj3MJ72PunwRbraeENHto5VmSK1jRZF6MAODWhkbdABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFAHI+OfHOm+FwtvPKrX0q5jj3AY9Cc/wAqxqVlDTqdNDDTrarY+Y9OszYa5rF3qFz51xfy+aJyNu8kkkY6dTWXtVUR0SwzpMu28byoDxyTkHrUgO2qOSOMcUmaRKVwfnOD2qbGlyJELknHGaa0C99i1HAcDIwfpRzC5blyONvu7cn2OPwqriSsxynB2/xGlcqwyRmHAPJ9aHqCdiCRieW5OMVFi7lV5FXqAGqyGU7mc7MZ460W1FfQq2L5uFwauJlI9A0Nt9qiqcvJw1aIxe55NrGhvd/EAoSux7tQzv0G5sc1UdEYzV3c+8NNtUsdPtrWIARwxqigDAwBitTAsUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQBFeTpa2k1xJ9yJGdvoBmk3ZXGlzOyPj7xBK3jHxpeXd5uk82bykx0UDrj2HSvJlNv3u59RSpxpU+RdDovEHh9rO3hgnjbynQNE7dQw56/lTjzR1ZyuSqJpGba5AXn5iOea6EcclqRzZJbA46cUmWtindeVaxCS4I5+6meWNNA2Y897qNwQYrbyouoVRyR+NXFRM5Sn0QkXiS5sZliuInZh/A6FavkizP2s1uja0/xXZXDmO5hNu/uCRWcqbWxrCsnozXjMMxzEykdiDmsdmdO60IXj2tgjjpWiIaIZ4iSSD/APWpFWMq6hkDZI4qiGmZV2sqtkjimiHdEMRKyhhxmmTe56B4ekCwIwPQVaMpmFY2txqHjXSra2WM3N3qEfzScgKrBuf++T+VaRRhUZ9j1oYBQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFAGP4yYr4T1gjr9kk/9BNRV+BmtD+JH1Pl/wyqWGlreyj94WfaP+BE5/lXkM+kk7touS+Jk1i8aDFwZEAJLnKg5xxVu71ZzuKjoiBRtLccCuiOxxy+IjUgNubpnpSZa7FO58hpt7IHfsW5xUttlJJCRTQzThC24qeQgLEflSVym0S69b2K24W5jlRiM5eMj+Yq1foZuzWpxr2qFsxvyOhHII9Kvma3M+RPVHRaBNsKxs3K/rWcjaGmjNvzxkKxHX0pJ2LZHcSqmct8oP6Ur6j6FSfUrXaVMq8dc8flVKMjOU4ozZ3iueUcEemapXW5m2pbELWbBQw5NarUxlodToAPlRrk5NUiWek/CDw7HL4nutTkQGOyTZHnnDsev12j9a1ic1RntNWZBQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFAGT4uXd4W1cf8ATpKf/HTUVPgZpR0qR9T5X1NJp4NI0+0JHmDA92Jryt3Y+jVrOTNKPTLXTYGijG+VGJaY9XPt6AVV7uyMJN2uV5/khHYtya6LWRx3u7lJyWYgGoe5pHYzdStLllLbyq/7Iq4pEyuZNrouoTQTLFevJuXEaRv5Wxs9eOv/ANeqUop7GbpzaumVINK1j+2obbU9RNvbDajSoxdQvXPu3bpWrlDsYKFRdSaK3dbwwQssrliEdAQsnXt2PtWTVzog7bnQafZOHG9SrqcH61ns7G61V0TajC8CElsDr+NNoSZz9/qrLuXdkEY60KBMpnOTyTztmMMWzn61snY5pJyD7JfAb0jlUj0OKvnizL2c1saOh6vd2l5Gt3uK5wVbuKLLoPmltI9a0nyGEc1rgxSDcvt7VJXQ96+HemjTvDEBK7ZLkmd/x6f+OgVvFWRyyd2dNTJCgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKAK2pwfatNu7f8A56xPH+YIpSV00VF2kmfL8Fu/ly5ys1tKWgJ4KtXj6rY+hum/JkM19NcWyG7wLosxkK45Of8AJrSCvK5hV92NkQ3Y3JnPyiulnLFdCtBnfwBnNc7Z1xVkWLq1dl+Rs8cr/wDroUgcLmNcWcsbkwz+S/cHH9MVompGbjKOxRGkXlxJvacNnuAa0vFGLU2XY7Y2S8ENIDlSwGVPqKmVTsaRpX3Zq6TbXDyCSQnbnJY5rNXbNmlFWIPEyvIjsvQDHFXfUhx0POpxK8pEcckrj+BBya2iccm7mh+70dYJ9QhWSOSJ5CA8hZWA+VDjGCTgZ6c1SSkRKUodCzZ+IY7hQixvGCAfKn757K2OfxrKVJo3hXUiwkUN8CU4YHpjlTRG6HOzO28OTw6NoH2u5RpYo3zsVsF+egPr1rS/Uwa6Hv3w58cWvi+0cR2v2OaJQ3lb9429ODgdK1jPmOepTcDsqszCgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgDwjxjDbaZf6nZNbE3U1y7rJjaI1JDBs9xt4x3JPpXmVEoSaZ6tFzqcrW1jgJvKa/aOBw4TlsdjRR7muI0Vhk7gQH1JzmtZGMNHcgsiWcn1rGWh003c3rGANwOpojqE3YjurOCP55SBn17VTSQk2yjLd2Y/dxMTheQtAyijRzS4gj2vn+Kpb7Gijbc0reWeOQGYHyyMdP8+lF7C5U9inq85MJ8scnOTTiyZRZw0tuRceYBjmt07HLKN2SvLMIykhLwHqpGQPwpvXVCWmkirNaRT2pgjuWjjJDbQeM+tClLqKcINaE+mrcWF5umfzUZNu8DhsdCferdnsZRutzrtXl8nwdZoed+9yO5x/+s1nJ2RtSjzS1Oy/Zb8248Ua1OSTFFbCMDPAJZcfyNPD3crjx6UYqK7n0nXWeWFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFAHHfEzRNLv/D15eX0JFxBF+7lRirA9AD6jJ71jWhGUbs3w9ScZJRZ856VbCEXjbTjPBJznrXPHY7al29SvfS/KoHbpTF0IrS5AkA7DrWc0bU5G3BqAhBJPbpUR0NZanOanq0l9eGCEnI64PStFHqyHO3uo0dPsfsy/a7nb9mX5WOehPc0parQqHuvU2LCws7qaOe0uoyG7Hjn69MVEUi5ze9jfk0svHM7EGONchieCaqUDOFTWxzt5HGuFkXORWcE+prNnL6jbtHcs9vGHj7g963uloc/K3qJBaxXUIlt849D29qlNp2KcVJXEbSoWctsAcdR0qnJkKEWMXT8SBV+6eCKqLuZTjY0vFISIWdqeQkDMR9Rj/2Wpm9TShHRs9s/Zu8Ky6D4Nk1C8Xbc6m4kA9Ix938ySfpiuihGy5u5yY2pzT5V0PW63OMKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKAOM+K92Lfwx5WeZpAuPUDn/Csa7tE6MMrzPCmTNnKR0ZsfpXLT2O2r8Rzdy/7xvagqxQtyWdnAwoNU9iY7lXUdQlmZrTT/vrzJKfuxj+p9qUIdWOpUt7sSxoqR2tudmSzNzI3VjWklczi2jc8xZraRZTuiddrDsRUpWZq5XWpzUFtPoszTafK/kNy0LnKn39jVOKktTOM3B3R1ej+J4bmyCvNtb7pQnp7VzTpyR2QqRkrlbXNZtkK+ZcJGVHAAycU4RkROpFaMzU1+2lA8rzSF6uEwD+dXyO5KqpqyKmjaiWvZlxgO5fHpzTmuoqcuhuTYLFj3qEy2hunbnvAp5BOAa1gc9Q1tK0STxL8RF0+bISR0iwOqxKAXP5A/nStzTsUp+zpcx9XQRRwQRwwoEijUIijooAwAK7tjyW76j6ACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgDyL44aiRcWdmp+5GZD9Sf/rVzYh9Dswq6nlltcbrORSejA1jDY6Km9zDmAEjE9KXUu90U3yqsgGCelU9SY6Mx9r21syIMtIxZz6/5FWjJ6FjRtTt5YmRnVHQ7Sp60pJlU2mdHaSQPgK/XjgVKTNWkT6hpsc1lIiu4Ygc7OBzVO5KimchcaKyucpvYdHjbmlzDdF9Cg2mlJTuDbu+7rWikc7ptPUuJEFwD8uBSLWg+LZb3UcgIG44J9DUS1RcWrmw9wSAM81mkbylY2/D8Y88SyH5U5rVKyOabueyfBrwyLe81HXboZuJMQRZ6qAAWJ9+g/Oqw8b3mY4mpdKCPVq6jjCgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoA+bvinq66n4inljOY87EI7gcA/jjNcVV3kelQjyxOJWfZuB4DDH41MTWotCjdSHeDV2MkyNmyAeKQ7iR2/nSF16Ace9F7DtzGz4b0rT7W+a5u9Oiu1miKlHH8XrnHBq1O24ew517rsz0ux8J+CdR1GKysZUS6jg81ooZTllOACfpV8sXsc8qlWkrSRVvfhpepbyPZ3wK72McTjGVzxkjvUuDNI4qN9UcBqnhrXLOJ7m40+XygCzN7etRZ9To9pCTtFmDOHQr58UkZbkB1xkU7Et6kNzGgi37hx79KNUZStuZt46yWrlBll5yPamiW+xt2ahwHfoo5qIo1mzpvCWjal4iWe00uAySyLg4IUIpOCST061dm9EY8yjrI+mvCOkz6NoyW95P9ou3PmTSDOC5AzjP0ranDkVjkqS5nobVaEBQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQBxnxH8Upoukz20Yf7XcRlY2HAHYnP0rCpVtojelRcnc+c9VlMzoc/wjvXMz0ImTeMVHHQU4hMoLOMYJrQw2ZNEQWOe/SkO5ds5Qsw46dalouLszetJlC44weR9alOzNvQ2LOwttVgYOis4XJ3DkepHfPvWiXY61UUo2krok0zUdf0m3WystbMEEUYSGO7hE6dwMMMMBjHXd0qlPozmrZevipq5uT+Pb+GNbfU9HtrwkKGks7oMjDgHhgMcZ4z+NW6iW5yrAVJaxVvUy/FniGx1G3ufs2n/vzFsjEoUct16E4xUupHsUsBWW7PDLnRLmS5aS5uZGUtnYGIXPoB6CnzmU6PL1NeCwACouQg5NQ5FRgaK7ivkgfM5yfp6UJWQpO7ufTXwY8OHRPDIuZ49tze4cg9VQfdH6k/iK6IRsjjqy5megVZmFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAcF8UfiPpngrTJkEsc+suv7i1ByVJ6M/oP59qpRuJs8Z+Ffxb8SN4rnh1i4/tDTLhMkzMAYJSeCv8As9iOlRWkoI0pU3Nnf+O5pPFHgG31OCL/AE2zf/SI0OfL7MDyOn51wTldKR20lyS5Txot5qKwOeKDoRDOu5Dmmgkc9eDyJwQflrRHPIs2sgc9frTFcvgFW3KO1SWXFkwBk4xzWb0Nky/p+uCylJkYof7w6fjVK9jSFRReprjVoZwHSRW3HoCCKk741o9CW4vLZkLOEXngfjTuaSnZbmHdXiYYREMM/ez0qkrHn1sRfSJhuRJLvboOgpnHfuNAKsW7dh60JEOXRHpXwj8BTa9qMepalEy6ZE247hjzmH8I9vU1tCN9WYVJ2VkfSIAAAAwB0ArY5goAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKAMvxFr+m+HrFrvVblIYwPlXqzn0Ud6aTewHgPj344apNFLB4ejjs4Wyvm/elA9c9Bn6ceta+ztuJngep3txeTyT3UsksshLM7sSWPuaokl8OagLDVoWkbEL/u3PoD3/OubEw5oaHThZ8k1fY+jfB+pNLPHbzxie11JTBJG7gRiYDl29cgKfqTXlJ30Z6NSNtuh5/qth/Zms32nlonMEpA8sfKAeQPyq4u6LWpA0Xy8jg1dwMHVbdSp/vDofarTMJIxbCcxTbH6g1oYnRW5OwEHOazZqti1sMkeUHPepe5oitcwuY/u5JHpzQtxvYypLJ4nZ4nkRz/dOK0uZ2a2CM3g/wBZOzj0NLQfNPqy3HI7ABiaZncv2sPmgn0ppEuR6P8ADn4a3evTw32qK1vpYIYZ+9MPRfb3rWMO5jOpbY+h7S3htLaO3tYligjUKiKMBRWpzktABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFAFPVdTstJtTc6lcxW8I/ic4z7Adz9KaTewHlviT4xQASweHoFZxkC4uXCLn2XP8AP8q1jRb3C9jxHxF4kv8AXHuJ9Su1efpufOSPRcDAFbJJKyEclp2lXuq6rBYadC91dXLbEjj5J9z6DuT2qQLvxG8Aa74IeD+2IUa3mGEuITujLY+7njBFZ3vsFjhWfNG4j2L4Ua+mqWv9j3YR7gFTGJOjuv3Pz5U/UV5dejyyutmelRrc8Nd0dj8SHF1caTqxeBHuIhDLbQocROOcFvXtjFYXuzop6Kxy9ymyP27VqUYt8mUO7kdjQmTJaHMX0DbyQRkdCK2TOWUXcsadf4IR+3Ymm1cSlY6Gwu4vLwSM/lWUkzoi0y8k6bP4fQVBrcjkVWODtye1O4inPCi5xwKpMhpEUMQZwF556Va1MZWR7R8IvAttqKNqWqL5tvC+2OL+F2HJz6gZH1raETlqSa0PcVUKoVQAoGAB2rUxFoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgCK6uIbWBpriRY41GSzHFFxpN7HBeIfGGqSs0OiwW1lF/wA/WoSCMn/dQ8/iRQ6lOHxs2hhqtT4Itnnd7oN1r0ryav4tsfPPtJLgfiAB+FCxtFaJmzy/Er7DM6HwJoFtLnWfFiNIx+7b2zt+v/1qTzCiupUcrxU9VExvF3hbw7b30S6XqV5c26r+93BQWPopxx+VcdfNVF2grnp4Th+rVjzVXynunwy8IeHdCsIb3RbMCa4iBNxI2+QqQDjPb6DArsjV9pG54Vai6M3B9DqfEeh6f4i0e40zV7ZLi0nXDIw6ehB7EdjT2Mj4R+KPg+58DeLrrSp9z2/+stpiP9ZGeh+vY+4q07iasc7YXc9ldxXNrIY5ozuUg05RUlZjjJxd0fSem6/H4z+Gd3Il3Z2EkREk8W35mnHLemAcBh16+1eVXpunLXY9GhUUtUcTLf8AmWiDbjjuMEeoNDZ1JXM6eQ+We49KSeo2tDHnUOh3VonYwavuY11G0cv3ua1Tuc8o2Ft9QKcOSCKbVyVJxNeDUlwo3Zx71m4G8aqZfGph0BB6d6jlLc0yMXhllCISc8DFaKJlKZu6HZz3eoW1lYqXuJ3VM9Tknp/9eq8kZvuz638O6VFoui2mnw8rAgUt/ebqT+JzXQlZWORu7uaNMQUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAQXt5bWMBmu5o4Yx/E5xUznGCvJmlOlOq+WCuzhde+IlvFuj0wZ9JXHX6D/ABrzq2P6Uz28Nkkpa1fuOB1LxHqN/IzNcSEk5yT0+np+FcLrVJO7Z7lPA0KatymE7lSSzFietR6narbRRWlndlIQ+X7jr+dLmS2LVO+rKpyvHOPU81N2bpJFW5OfYU7DTsex/BXXjdaZJpkz5ktDmPPUof8AA/zFepgat1yPofI5/hPZ1FWjtL8z1QHIr0T5o8t/aB8CL4y8HvNaRbtX0/M1uR1cfxR/iBx7gU07MrdHxVgoxBBBHBB4INakHoXwO1eWw8bRWkMVs7aghg8yc/LEMZLfkDXPioc0Lm1CVpWOp8V6S2malOvnLMDKyyPGuED9cDr1Bz9Q1eYnpY9aDOflbHGapFspzYIxVJmbRm3AD8EZrRMykrmRdwsG/ka1TOecBkG8HvVXIszTtEd3AY8elIdmb8UaRKBEgB7nvUORoonuH7P3hoPc3GuXKZWH91Bn+8R8x/AHH41pSV9TKvK3uo90rc5QoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoA5nxd4pi0aMwW+Jb9hwvUJ7n/AArjxOKVJcsdz08Bl0sS+aWkTx/XNVury4Mt7K88x/vH5V+grx51JTd5M+uw+Hp0o8tNWRjvMI1Mkzc+gpW7nRa+kRUuNwxjaD2zUc/Yr2XVkb5bviluWlYrSDFMtMibI6UFEEyj2q0Sy74K1ptA8T2l0WIi3+XKM9UPB/Lr+Fa0qnspqRzY7DLF4eUOvQ+obeQOgKkFSMg17yd1c/OpRcXZkjgMpB6HimSj5K/aS+H6aJqf/CQaVAVs7pz9qVR8sch6N7A9D7/Wrg+gSXU8Rgla3njlUurIwOUYqw+hHSrkrqwk7O59F64Ytb0XTdT0/RksNJ1RFg+0MFDiccRORgnG75SeuGPrmvGcHGTTPTU7xTTPK4tQWWaW3uI2t72FikkLjBVhwRWsqTirrYunXU9HuOmbjrUotlSUg9ODTRLKciZJ4q0yGhiREN6U7k2NK1+UdhQwSNnTl82eNFGSxwB71OpeiPsPwZpCaH4ZsLFANyRhpCO7nkn867IKysebUlzSbNqqICgAoAKACgAoAKACgAoAKACgAoAKACgAoAKACgAoAKAOT8deLbfQLXyklX7ZJwqjkj6D1rixeJ9kuWO56uWZdLFS5mvdR4lqurXU26Zm2tK3GWyx9ya8KUm3c+3oYaEfd7GTJcSFTlzn60Js6fZR7DEc5DEbz2y3Shu4ciRat5o5SdvBHUHqKViWmiRpArUE8pFIyt061aE00V379Kqw0yNiNpFNDZmXQyc96HqODsz3r4M+IDqmg/YriTddWWE5PLJ/Cf6fhXqYGtzR5Xuj43PsH7Gt7SK0l+Z6SDkV6J8+ZniHTLbVdLntbyBJ4JFKvG4yGU9RS2HufFnxg+Hdz4H1gPbrJNol181rcEdPWNj/AHh+o59a1TuS1Y6L4U3Wma/4L1bw9rMuoXl8ufsVpEzHYgGdygdcN68DiuHEw5Zc6R2YeTlHkbOW8awPqmkWviLyjBqUL/YtXiKhGS4X7shHH3xzwOoNa0Zcr5Oj2MqibXN1RztlrbqvlXPzL2fuPrTqYdPWJdPEtaSNJpkZQyMCD0INc3K1ozqUlLVDBJkdaVhiiUZosK5bhfIGKYHU+DJbW113TDfH5JrhYU/3j0P0BoabTsS5KJ794b8dw6XqZ0vV0NvYMoa2nJyF4AZT6ANn6fTGJpYjlfLLY6quAeJpe2payW6PUIpEmiWSJ1eNhlWU5BHqDXenfY8Rpp2Y6gQUAFABQAUAFABQAUAFABQAUAFABQAUAFABQAUAcX4+8cW/h2NrOzAuNWdeIxyIgf4n9PYd648VilSXLHc9fLMqni3zz0h+foeJSTTXl1JdXcrz3cx+Z3PP4egrwpScndn3MKcaUVCKskZt/cGa6IThE+VfpSsdFOPKiM9KChqt6UAxHwTuzhh0YdRTESwXO4iOUYk9ujfT/CixnJWHltrYP61djO4Fgw4qkTYjHoaTKTuULz5WI7HpQ</t>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAbAAAAIcCAYAAACXePsiAAAgAElEQVR4nOzdWYyl6X3f9++zvctZqk4tvU53z86lh1rIEUVLocVhQMCBrUQOIgq2ciHmIiYgOBdxgPguEGEEufGFgVhxYN2ICHSRyFcWBETWRokSHYocSuSIw2W2numZXqq7qk7V2d7lWXLxnO6ZOBwPnVhT3eX/B2jUMqfOeee8qPrheZ7/839ACCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIYQQQgghhBBCCCGEEEIIIcTDTJ30BYh/v/6r/+G/PulL+HfmqgJdWabzOT/3N/4WL37zBV5/6dUzF0dn/+mzV3/sFz76489y4ZELrHxPFzwhBryPeBLOWrTWgKWwBYW1DMsapxRd59FaY62m7z0hRKw1aK0JIdL7npQCZVGilSKlhFIKrRTqnb8aCUgBtIaYQClIiagVCUVHwseEBjzQ+MB8teTu4ZT9O3fYu7tPXVY8/YGn2Nrc4K2bt3ji8iWsUgytJbQNv/O7v/UrEL5w7fWXOTy6cyL34f32P33hn530JYiHnD3pCxDiB/j5v/e5z//qpd3zZ2sKbt+4yVe+8hVuHh9yuH9I13UopUkkuhBQyhCNoS5LNocDHjlziSuXL7O1vc2wHlDqAozGGEMEIqCswWjQyuV80hqTIISQw+tefikFKQIqB5nWoBQxRVJKxJTQWuGMofOeVdPyrRe/w93pEfPVAmcdi+WC/bv7XHv9dT7+sR9ntLnJd19+hcloxEZdc+ncGT796c/8yh/+4e8AfOFk3nIhHj4SYOJBcgb4p3/ns3/3F1Qb+MtvvcDtN25x/c3r9CGw9A2tD6QUiTGBVhjraOYNR12L0Yau99TJMByOGQ1rdnd2uHzlCufOnOGRK1fY2d6iMIaiLDFKg0qklAAwOofc+kvu55hS90ddKAUhkBQElcOw7XJw/cU3X+DO0QEBxWy55NXXXiWEQOkcg8GAQTXkm998gY99/Fma5ZKuqpjN59wpLNuTMT/5iZ/6lWuvv/xt4F+cyLsvxENGAkw8KH7+v/2lz/+qHVRn/+Ib3+TGK29wcOsOdAmdFE1oCOtkSQl850FpymJITCtWbY/3C27cvI1ThrooCSnRdh1VWXJmd5ednR1G4xG7ky0++PTTPHrxIme2t5hsTqirkmAtxhic0uvXSfdDLAGRhAF8COjC0cyXzNuG23t3+e4rr3D99essfctssWR3excVIsvjGUtgMZuzu73Na3fvMhqPKIqC0Hsgcf3N1/nI1Q9y8fwjfPQnfvJX/+D3f/uPgb2TuQ1CPDwkwMSD4Oc+91/84m82bcdLf/Ei1199lflsxdgOcNbQrFpqNwTvib4HIq7ULGYrprNbpJTwPjKbrQDNtO25ezRDKYtymg3lKGYLFo1nY2vFWzdv86///JtsVgVnJ1ucO3uWJ596iqcff4IL586xs7W1XivLa1wxJWIKBBJaGZIxtG3PN/7yBV57/TqvvvYauiiYrVYYoCwKXnrlJYqiYDAYsLd3F2Na9vb2KIqKN65dY2uyTdd1HM1mHB8d4FNg8omP8+TTT5998S8v/OrR/O5nT/ieCPHAMyd9AeLfr49+6tmTvoR/V6N/+Mv/3W8fH803v/bVr/Pmy6+hPThdErtA1/ckEgnwMeFjIIRE3/aEEOl8wPvAbLXk6HjGqutZNQ2rEDDOMBmOUUaTtFoXgETiemSlgdh13Lp1i2vXrvHKa6/yyssvcXA8Yzaf4xO0MeZRmNEotV7/Al67eYM/+9o3GIxHbG1vc7xYMpvP2bt7QPKejeGQw7uHzI+PsMqQfE/wPZONDVSCGzfe4jvf+z5H0wNc4VApsn12h7IqwPurN26+/kVgerK35q/WH/7uV0/6EsRDTkZgp8zZRyYnfQk/tI8/8wkevfTYP9q7fefyd771LdrDOZNqg6736ACdTnjv8aFHKZfDJyboIylC7wPee+bzBUeLGc1yRdN2LHyPtRatdA4erZgeHaG15ng2A8Bpy9BZdgY1rijw3pNSous6/vJ730MBo60tPvjUk1y4eJHRaMTZ8+c5s7sLwLdf/B6vvfE655sWrxRt27A5HjObzbh58yZntnZIvqPve3o6lFKU1uKbjm79UXUtXegZXzjPqy+/yoeffopzz3yQS48/xb/87f/jOeDXT+reCPEwkAATJ+ljVhX/zfPf+jpHtw8JK4+1BS4ZIhGdcilgrp3QGKVQIbBsG7q2ZbFsmS0XHB8fsz87ZtX0xBhYERgoje87lqslg3pAiBEfwv0y+aKwhD5w5+4BmxsbObwirDqP0ZoA3Lr+JnsHhyilMEZx8ZGLjOoa7xPLpiGlxPW9W2iteeXVV7HGsLmxhUYRY6TznnbVoazCGsPxsuHoaEY9r2mWDctmwSMXzhH6nrZpeen7r3DhzBkuXrjIo1c+8CkkwIT4t5IAEyfF/MzHfvqf/8EffMm0i4bYR3bHE6bTY6wydDGt93AVdCgMhhAiMUHwnuWy42g+YzabMZ0ec7BcEL0HrXHGoDtP20foAjYptqoRMUZa3xFCwPc9SimU98xmM5ZtS7lYoY1BVY6drS1WXUsfItrlmfbmjTfx3tP0PVopxsMRi+USh0IlRdN1dO0daFs6t6BfNKyWc4IPFGVFVRQopfDLluV8Rh88cdUw3bvDZLLFctYwO1oxfGLCk0998LkXvyVTbEL820iAnTLfv3HjpC/hh/KLf+vn/v43vv/iswcHhyyXDcOqpmkahq4k+IhXCaUVXoFJkdAH2q6n6zrSer/W0eERh0dHLJqGtutyqaBK1ChS6DDG4kPPCghtD1phUeiYiCZyr1p+vmyIwRN0DjBH4vD4iD4lVn3P6rClLC2zxQLvewZFiVKaXMmvUc6RfGA+X6K1Js6OMesnL13JvJ2zWiwIIYdmSokYItujDcZlie4i+2++xdA4hsMxIcKgHD8GPAZce//vjhAPBwkwcRIuPf3UB//Rl3//KxjIJeVNICUw2uAN6BDodS6YgEhQii5G2hDoQmTRrtifHTE7PibGRFo/kgSh9SilsbUiBWiXC9rlEusKytJhtEYFTQtURUEfPM5YEjlcFt2KaDQxRla+ZVgPqKxjtWpYNCvcEAyKRdthtWYWI4UtqccV7dEMpRRdaFHKoK2mqB0+BNquo2lXKKUYDAYMRwOWR3PaNOfmwSFbW9sMxgMi8OSHrvLHX/md55BpRCHelQTYKWPdg39Lf+4zP/s/37m9P04+smxWBB+ojSVFxbLriCHhyZ0uUoq0KrAIiWm7JMXAdDVj2i+ZxY7GAU1H0UdMaTEpolJEaUXXe5wp0EqvR249mBLnHFZZVNJ0q5boPQvVU6WasrQs5nPKlOhVrnq0dUUVIqvFkrLzVFVCO0PsPZH8S1QqRVoEdAq0KrBqFpRFgdYOaxU+BGJsKZym7TpS39D6Brqe2WLOmQvbDDcrumaB1mcYjze4fTx/DgkwId7Vg//XTpw2Z579kR//29/8+jcJbQMoiqLERZ2rDVForbBGEYj0fsWiaQjBkRL0IdCHAEANpBjpFHgd0TGQQiLpgA4GRSLh8UmRnMMDsfP0PmLVemUtanoi1lhC8MSg0Qli32OsYYhGrRpWykNK1FVB4fKG56gUy2VDUa4rJH3emNy1K4wuSMnStg1t15JiwhUWpXRuPVWWKAVNt2C0OcQYxXg8pCgMs/kxg7LizPaZT8X27gneKiEebBJgp8yoGpz0JbyXq4fHUw6Pj4ke7jUdzJV+mrKwhAht9IQQiH3e5xWTInlPs17viiGy6nrariP0PSlGDJoUIwGFMkBKhBTRUUP0eED3Hm00aI02DhUNkFAq0jctOgWctRACxui8phUDOiVKY6jLmsKYXBFpS3SV6Lwn9IGQIhAotSG2HYu2g5Twfn191lE4x9Z4TDWsKRI0Cvq+4YlHn6Iwmq5ZMT5/gUDgYx/50ce+/vwfXABuntTNEuJBJgF2yjz96OMnfQnv5epsekzfeZQyoBKk3LZJa000iRQ93vd52k3B0FmOFoHOe/q2JcZI3+cNy7HvSSnl4gyjiTo3foooUlL0EZQGazQ6RAqVNyQXxqK1oY8BQx4VBd/S6UCpCjQKHXrqcsiwLMArYkw4Z3Axv4Ixns3BkNVySRMiKIPF4SpNu8wFH0ZbglEEE6kKh1KGAoVatcy7GQXQhYaXX/kujz5+hcsXL+CcQ/nEx37ko3z/O8//BPBbJ3zPhHggSYCdMo89+AH2keWsQcWEMQa0xqSE9qyPN4koldAaCAkVE51P9OugcmVJ1fccL1fEpiHFhEm5U0foPT5GXFGi0SgUBQYdA8SABSwRgwJ6rArEFHHaUWmHVwmnIkXsSSFAzAGr1ZhqMEDFSIoBEyHEAEmjVGRYWkodCSlQ2gJDYHM0ZF0Wef9/3NrcKHjRLOhaT1FaCmtZec9jj17mZ/76TzOoa0iRyjrGo026xj+LBJgQP5AE2ClTOnfSl/Berh7fOcJ7z2yxZFKNsNbhmxUh+Dw1d/9vviIEhV91rLoWh2KxWKJ84Pbdu6SmR2lF0oqKvMnZKQVdoCh0PsMr+nzeF4G+7wnJU+g6d6InUmlNZRWlVsTaMapKFApDPhss+UBNZLJev2r7HkIu4khaoYgU2jCPnsJqHBHnW2pX5nJ/36F0PrMs9j0KKAE7HKAKl4tEkqYmYqKn65bU9RgfAnVZMyg3HrreYEK8XyTAThm77qT+AHvGe4+KMKiqPAoDjMml7YEE4d/8EYVJCt+16JS7YDSLBSnlUZKNkDSg8/EmhYYK8CSIEd23FEYzchpMSakV1q1DJSVsqalsQilNaRXb9Yh6VFEPBoS2x/ct42FJ5QasVnNCHymqiuA7Vk1LuzzibD3EGUOKgboYsDmqMEZjlGU4HmKtZT5f5EMzU0Ktzw9bdi3TeeTVb3+Tr/zR7/G3P/tfEosBXduxubHFBz/8EQkwId6FBNgpU5XVSV/CeymM0TitcFWF8rmnoSMRVCLFSFQReMehXChKbWj6HmMMXd/jmw6AlAIak8+cBKwG+paQejRQFY6NQUXlDMO6xDqLiYmizHvCdFXirMUqjVUJaww7G5uMJxuMx2NUiMymx6gEVVXRlAarNYPRkNVyxWq5ZG+vxaSeunRsjiZsj0t2xiOctSilGA5GuKKg6zqM1nnNzjlWvefO0Yy92T6v33ydr335j/jAh3+MZ3/6UxTGAQqt7db7foeEeEhIgJ0ybduf9CW8l2skfsxYC8mRYuDekEurlEdg/y/q/mhJxUhsOkLb4kxe6bq3zGQARaI04FKkcIad0YDdMztsjsZsjIeUpYHeUxY5wFTpcK6kLhxlWVBZQ2kthXOUpoDk2XC5IKQqBoQQSSlgjKOxCrOzycWz20wPplTDmgu7Z6l1YDIaUzi3PrFZ46yl2BxjraVZNlSDEu0slx+7zPFqwejFgq/8+df5k9//Vzz59FU2ds4RIpy/9Njh+3VjhHjYSICdMg/B+TjXkg8/5qwjdJB0DqdMod5eAHuH/D2nLIvQ0fsegieaAqsMSimszvvHHImd4YDJ9oSzk222J5tsjocMRwPGZUFVuhxAKJJRYBXGOCqrGQ9qKldgtcJqB6FDRcemG+N9QGHQpSMmgMTuaIfjoyl6OGCrKqmqgvF4zEgpxrXD1gVG51EYCpyzxJjQXjEZ1FSDIbEcYAaXKQclnUp878abfO3Pvspn/uZ/Tp8A4yTAhHgXEmCnTN92J30J7+WaSoFCW5q2IabcuT3EmMvp0XginVL0CnrU/VGZdoaiMxiV6wn1unQ+xYgxoBQYDVujER+4colHz11gvFFTO0tpVC6BN3kKD/Lj3XoNTgMDpSjJJfm1NWALNKCVofcdMUYUitWqwQfPoKoZn5nQLxtAY6xGNXPq8QBrCiyR0imsye2rtDHMF3MGpWW4OYJ6gNEW6LmwNeGxyxfZn8/4xle/wo999OOcuXgRnfpTfSaYEP9/SICdMt2DP4X42ng4Rq0CDUs0ebNwbywBRYzQa4gq0KDxCoJKqAg6aawqSCl3y9A4lLYkv8Qqh1KecVFy6dwuT198hLPbG4wKQ201ioDRGlTKx7NojVGaCpMLK6xmVBRYrVEqUemIMQUAWkdCURCCR8XEpBzQ9z1t2zJwGsYl7XKFjj1FWTI7nhJjz1AN0XVFUThSSqyaBV27ZGuyA2UBvgNaGFdMTMHl82e4cfMO3/r+a/zx7/w2/9nf+btsWPZP9nYJ8eCSADtljo6PTvoS3su1TTck+YB1hoQGnxvnxphARe4Vbiidz+6693VUsAxtHkEZR6kURiU6BSEFCq0YjQZsbgwZjUqMUYTQ49EM6xK9nmaEfLaYNYZSOWLqMMZQVzWFNqTUY22B0Yq8PqcpjCZoTQgBYwzWmByIQKk0mzs7HB8fo5XCWkPfdcxjJIZAWy9zcUpMbI4nFDs7UBQQAsQIXQdasbu5ycUzu9w6mPH817/OX3vu05CiTCEK8S4kwE6Zg729k76E93Jt49ITGKPyH2+tSPrtwg11v7VU3oislEZZQ1AdSrE+OTni7L3VvoRVisI4BoOS7e1tzp/bYXMyprYaEzy1tVSFy+tkyqCUQxmNMYpKa2IyWG2pygKjFET9/wg7UkBbjRvkEVmzWKKNYmM05Hg+p21XFIVla2uT1WpFNR6sAzmSUqRrGpTS1KOaajjI+9OaJRQlWMV6UY0CxdZ4g/Pb27z62gu88p0XeezJKzKFKMS7kAA7ZV6/ef2kL+G9XHv68aehj/RdTzKJpHIhR94TFteFHAqj8vSi1hafEkpros+hh1b4mNAh4ayiKksmG2Munj9L5Qwx9ChjqaymcIbC3GsfVZC0wRiD04qcgxanFEZrYuwoqxxU93ohpmjQRpE0qBiphjX4gO88k+1N4qpjPp9TWIstCgptoCqw1ubN051HO03tSnAWvAenIeQDOLEGCke5arA+nxP2xKVHuH3jBheunJcRmBDvQgJMvN+OjhbTaxM7eswVhqg1kXxAZYyBEN8xGlN5d7LFMCPhVd6cHBV4DcSIjwpnLYPCMBoN2N6esLE5ysGlFYWzlMbkTcVGY3Qe1RltMRq0CjkkVSQpn1tIkfehKTRaKaJSxOBJaJzK04/BgK40JiZi5RjFITHkpr8xelQbCN6TfKCqCjbGmzAagW8hJRht5yAzOn/UYEJAxYCOkdF4yPRgj+OjqQSYEO9CAuyUeeYDHzjpS3hPy9X8S1XF55QFay3HR3MGoxF9N8daQwgRjEFFBUnRxUDSmnm/IjlF3+dClZQCg3JI6SJFUTIZjCiNZVitu2BoTeEsVueN0+V6lJe0wViDswqz7rxV6BKI+HXoOWdRKHzwOCLRWmL0+OCx1qJVIvY9ISasNQw36renDX0EImXlqIoxyjlwDkKfR1spwfEUhkPwfW5o3HUYBXVlsUqxnB6TVCRqWQMT4t1IgJ0y/9dX//SkL+GH8aWf/dTf+NxkY4vbd+4yGA3wvacoSlZNmzf+akWvA1obivWUn9Iqj8J0bqprjaULLZrE5mjEcFDTty2+7fLaksnViipFjMrVhXpdaq81WKcx63PAfN9irKaq8wGYKiqUThRK5VFf6FFaU9j1mV4konN51KU1Cii0JimNdoBRFNUgB1eMEAOQcj2KXodY14K1+WvfE7uGQkPbLjg8ustscUgxqCXAhHgXEmCnzEsvf/ekL+GH8Ud7H/4oTi84d+ER7h4eUFYV08UxhXO0yQMBTd6rFbTODX5TIsTAIvSk6AlaAZZSGapBhXMmnwcWAhZDoTVWg1MKq0DrhNYBrUHrvAE6d75XpJCIKmGUJhGJ0eMwaKVJRuNDRCsotQUUSedQTCa/pk4pF51oiMmjo8pVhqi81mVMDquU3v6tCyF3zIoeQk/wnuA9hVa0oWeROu4c7UuACfEuJMDESbj2ne/95Rd/4qOf/KX5akFZlTRNux4Nrf/ok1eicsm7pm1bmral67s8ArIu9zQ0msGwptDr0njnKJSj1G7dBSOvfa0L8dEqgtYo6zFEUlLrYo38qxCTJ8aIYV1ArxVWG5JKKJ07amitUEmTVCLGhNHq/uZorTQGS0oxj7zU+kAynRtdERP0fr3r2kLoICSIgRA9XdsSNGijmM2O2J8fHbzvd0eIh4QE2CmzbYcnfQk/lGuvvvrLj1586uOT7XNXR5ubWGug0DSdx5DyUSVKrcvZNWp9dlgukgjEfJwzpijQLo+UNFCrvM6V21OpHCSsu2+kvG5mksqnN69HYVprCp1PCQvR50MvbS7YUCi00lhn6OK6Z6M2qJSIIR+8qe5VS6p8jWiFSiFPH2qdR133GhQbDSnm77FegFMJvKfpmtztQylMUdD5ni4FGYEJ8S4kwMRJWX7pz/7os5/59H/yNTo1MKZg2a9I62k5bTXRB1Se70M7TUGiImH7ltR1NMOCSKA2id4l6mGNcxpspNUeSyQmS4whP29SpKSJUZGiwqTcfd6isfd/FfKxKioGjK3WIyuNUoqSQIo9KqzHZxEcBqNNrphchxc2t7pC5+cjrdfAnM3t8sN6LYwOlMmfu3w6dAiBru+YHx+TUuKFF16QABPiXUiAiZP04l986/lf/sAHPvTrZy9cYLBpCcGwWHqijihFLplPEZMSjkitYAzsm4Qy0ChPNFBazdBaKqPwYUWMhmgr9LqEXiXIibLu7BGBmNAxYY3GrHsIa13gvaf3+Tm1MaS+B2XBWVR0eU0rpNwGq7g34vV5qtAU5D5X6u2XSxGCyuGl1XpEtv7+vaIOZbDGEWPuRFI4R0qRsGrHQPO+3hUhHhISYOKkffHm7RsH1tp/cub8uSdWiwWFKfFW4SxUzrBRFvRG0zuHNY4tU3OgDSEkjE8MI1ReUfQBVzoKbamsuz8tGEPAWJvXrhTc2+cFee0pGZ9zRGkUCe0UWoFSCXQOSlTIQaNzaT+sPzdAiHltSyUwCcpyXaxh85RhiJD8/ewkrruQQL4GDXhP5SzK5arIrg8cTac0ob8K/NH7fVOEeBhIgIkHwW999/sv/J73/T+syvq/d2WsK1PgU4+JHZWODJxF2YKFKxmVJSNT4fuOpCI1iiIm6DxFhNqWFDqXw5PyqczK5YpDyNOSySWUTigipEBal82DwpQlpijWP9uBK4AA/SoXXxQOos7FGD6ua/IVebpw3d8wrqsN9brlVXLrta+YR3NqXcjRt+ATNA1aaepxjd23rJoFoOi69hkkwIT4gSTAxINiBfzKjb03/rfdrfP/xNnyZ5UBWwQan/d1aeewzlCVDmc0AYVRKh9Jog0pgVZuXZoesSbvISvWfRPvF3SoXOVnrVl328hNeZO614lxPQWYyOFkIPdEXJ9bpshBFbr835XNZfJa5a+JOZjuTSWmyLqRY/5ca+6P4JRaj9ASicigyi2xNLC9tc2Fye4z7+M9EOKhIgEmHjSvAP/pW7dff3Y0nvw9a8pf7GhGnY14l/JIxyWUg9jn1lM9gTZ1NKmnJ2CVwaAw8d65X28fmJkUJKVBaZK2aGWI65ZRQedfiNg2aGPAuvXerZBD5n5AQa4oNDmU1L31rnWRRl3mn1HkPV4x5GIN7/Oozun8M8qAcrlC0RXQ9xhtKJyDZsWwLLiyDrCrtWa1OF19ff/Hk74A8dDT7/0QIU7E88Dnbx9cvzBb3v18VO3zuk4UVaSoDJPdTWahpVWR427F3W7JXCWq7QlVVaJioo95StCnBFrjlcKjWfrAdNUxD5F5SjQp0aLpkmIVIgvf03b92yOmyNsVhvdCyLpctKF0PhrFWiDlzcnTo9w2aj6FxXEu+lgt11OI5ONTug5WHbAOMTQhJHTK3T8mg5ptZQm3967+zacf/PZgQpwECTDxoJsD//zu7dd+3nRz6jJydnfEh568xPZWQVKJZd9ytFriNsZUW5t0MeJV7p7R9J6QFG0kh1OCYApSWdFiOFz13G09s5RoTMUKQ69KGm1Yhki76tYBZqDzrBZzWCygaaHt88is6/PnTQ+r5u0pQ+sABa2nWyyYTQ9p5nNCr8AOoBqDG4AP9CHmBsNKY2JgnBQfOneBj19+8gzwvwNnT/QuCPEAkilE8cDbKXt2rpz9mYNXr7FTTfCqpzLw1O4u3712g2Y2Q+1sM65qVDRAj9UaHyM+RtqYSMFjyhptCqaLJfODY9CGuhxS1RWL2FPZRFU4RlVBUoo+BubNDJqOqjAYAsoHVitPbXsg5gKMrifqRDQarKXteqpyQMLQ+YAPnjZa2l4xuztntrxNWY/Y2d1mXDiMCnlPs8rrZaujKWF2xCd+5j/m2Q99CC7s/MKljeq53/3an/x94DdP9m4I8eCQABMPLL3/Imfe/vLT58/v8NMf/SS3X36LP3/+W5wb1OwVmh5NPJzhF03uFB8Vad1gN6FofGAw2KAPkcP9A27evsP+4SHKWcxgSFE4diebbAxqbIxsDMcURlMaxWq5QIXARmnZrAsKIHU9pgsU2hF9h9f5qJfegFeapXEc3dnD+4guKlarFXf3D9mbHiGuEAwAACAASURBVLGYdxzPZ2hXsLO5xU6ZePSRs1x+8hKDYYnpIxWK3fEGzzz6aK50fPU6rPbPPnnm/BeRABPiPgkw8eB54ys/aL7suU997JM8Ntml3FjQP/kEpa25c2OP/dkS3XaErkN5T1IJHwMKRQC6puO117/N3sGU6fGMo7bheLGgjZGAonIFw+Egnx2mYGM0gtiyUVXUrmBzPOTcZJNVXTGyllJpjHUEevq+QztLR+SoaziaL3httmLa9BwfL5gtlyxWPas+slp1JKUxZUlpA/tHS84PNV2zQBeKxx+7hLUWReLRc2epds/A/Bhef4XvvvEy9qnH99/3eyHEA0wCTDwwLrTXuVAB1cUf9J830u0p8xstl+yQfrJL5UYc3r7Ll//0ebYGCq17pu2UcVni+5aiKDDW8tJ3XuKP/+TLdEkxXfUEUxKtIfSe0ahmb9GAAusM47pGaygNpNixPRpw8cxZ3OMfwHbQO01Foi81hTXEFInREKzlzmzGd195lVdv3GJ/uqTHMGs6Vq2nHm6gjGFUF5Rtz5lJwc7mJluTLQo8se0Z2QI7rJge3uXM2V3olrB3g+baK5ztGkLv997nWyLEA00C7JT57E9dPelL+P9ma/O9HvHS3vXrn5jdbXn8kafYHI/QOxt88pP/ETdefplp27CcHeGGFSoknHV0XcdisSDh2T23S5sMw2jokqZTmtj36K5jY2eTpm8Jvme2aiisgsIyqkvquiJGz3I2p3UllXI0qcdojdYFXehoup5lTByvWkJSKGVBK/reo13Bxnibejyi0IrJeMjZzSGPXzzPeDQiJgXdinFVYXXu2uG7DmeLXMHoSqqtHfo3XqNIWjrTC/EOEmCnjDOntrD0ZUL8xGJ2xPHhIcpa4kDx5KOPc/XqM/zL3/sKgxtv0bYtuqyx1tL3PSEEJlsTfvRHf5yjRUNRb6LHI+ZtT+wDJiXKekC7amnbhv39u+jYUVnNZDRgUhU4q6lKRww9TddTWnDFmLIsCS3E0NG3PfSRwtZsbG/TlQP66RE+gKsd2uamveWgZnNrizZ4ztYlg2KA9iWTcZmb/YZA5SyFtmALmJTwpqbe2mZlrUwhCvEOEmCnzGK1OOlL+Kvy0qXRJnYSqYzGOsdiuaTRx3z82Wf5s298DWstoDHOkVLCOQsUwIhhlRhvKjCOw1VLXC5pu47D6RGrxZLDg0OMtagU2BzUFKMBDgidp1QWEwMxNShdMtnYZFCXBO9JKWF0QYodfdOzms84mB5ysGrZu7uPT5qoj/Bdx5VLl3hrPuXg9Zd58rErlAou7UzYGg7YGg6gKqBtSSGws70DW2dySX41xIbIsutlClGId5AAO2WO21PbuPzlaEps4RgOh+yeO093sM/0+Igz4wnPfPgqr66OMUqRlCLGSFmWuaO9D3jfM9aW24f7vHntTaZHRyy6nht7+9zd22MwqKnKiuP9A65+8CrToymuXXF+d4udnQvUFkoLVWmpCktKiaZZMhptAi2z+YrY9vSzFakJPHXlCcaDES+/+jqF1WyeO8tzP/XXWE73+d4L36SfTlk4Tags5bDE6ZRbU8WAIfcE5vAAxhOox7TLOdNuKVOIQryDBNgpE9ypvaUv9ViSUdSDkrosOLu1hVKK5bzhicef5Ftf/TKhaYmDGmM01uU2UMVwwLJtmU6nTPduEedHxHZBqR1//Sd/khvX3+SN69eIKfGTH/sYP/HRj3Lr2mukboXqekwM1EVJWSqGVc1wOGRrewLqMqnvYP+Y+XHDxqDl3NaEzTPnoSqZaMfju+cBSCkx9D0b9YCrn/kM2+MRyffsTAbsbI9hsD6GxShqV/Dma28w8Jrdqz8CwwFl/QjTm9dkClGIdzi1f+3+Q3XoT+8IrDFDtusKVzqa1THdqsWvVhzfPeTM5haV1rn/rjEok7vPW2uoqzI3AFYKHQNbg5pl2xPQjDc22NCXuLKzRQDO755hUhYMHrlEqRTOJjbrio1hhbGRqiyoqhLqIQxHqHnDaBEY1iWaCZvjTZqo6UOESW7ioZSiKByjQcWgLBhWjrousQqqjQGU64bBsYcIpbEkbXIvx6NjGA/Bjvju175852RvgRAPFgkw8bA4OEz984/v7jwbrWa+mHE4PebO3j5H+wv09jbDomI+PSbtbqONxVmHc47SGkqjGBYFk+GQ2dYOXdcRIxRFxXJjTEKRUsJaS+h6qsqyUVdUhcVpKK3DWhhVNfV4DMMRuApsoJpsMD4+xAF959FtoIvrZr5aYY3B6UgRWlSI4D1lUeJGY6gqMBHs+nBLEiolRlXNwBTQLPNrpY7rs0MZgQnxDhJgp8x5Oz7pS/grc0j6tTSsnkWX9IsVwXdUzrIEBnXN5Ucus5zNcnjYClsU1EZRGChHFcEH6qKg1HB0dEy7WGBXnjEajKHzkdg16JQg9Rjl8uOtRamE046qGkC9AabMfRCrCoxie2PILEU6qzEmsFzkAyuLyoFRxOTziNBZbGlwtYVhAdqCjqD9/VOax+MRBYnQt7l5sFbcvHGLpdUSYEK8gwTYKTNT8b0f9PD6jcNm9Y8vTzZHzVGDDx2ESD2o2N6YsDkYcePgLvfPOk4BbQqMgaEr8dpTaEWhxpRK0RlLN1vSpo6+iTilcK7CGo1xNYNBxaB0+aiVGCmKgmpQ5ya964MyKQrwHXpYMwoeo0bEYLg7PaJpG6xT2NJBoXGFpd6osXUNGyMoHQRLnmiM4FtoO8b1kDol/LzJraSM5eD4gEPvZQpRiHeQABMPk/lhv/yN5NznV74nxUTbtGzvbHPhwjncSwbTBUqjUSHSty1BG3RR0KeI1aC0Iqp8cOSGKwhFSR8jMSm6FAkh4ooCYzRaJ6wxWKsBTVnWGDfg/iEOxqyPVrGwuYOJPTQdejzg7KDCdytWXYOxmmKcR4SUBqoylzTGCEmxnjskxIj3PcvlkgE1dTkEa0BpDlcNKHX3pN54IR5EEmCnzHk7OulL+Ct1B37tlvefH0zOsTx8g8nmFuV4QGcazuzU3Jm9Sdm1jAY1YX12V/KBaAwYh9UGZx3B94Rli7FDXIIQIrpt83ldJEajAYU1eO+JMaK1pq7t2yc1c+/ASwMkiB0Mx1AsQQWwETscME7DfOHK5Mdqk3/Wawgpf20NtCu6ZPA+0HYN075n99yjsLOF73turfz/ST61WgixJgEmHjbPT1P/xQL1S4PhBs1sQd972qZhczTmiQtX0DHSrVpq53BKAwodE9YonLEoA2hD0JYUIyEEYgiUpcNYQ1lXEBPRewBCCBhj0Hp9knLKJz2jdT7AUhtwDopyfQKzB5VL4u8dVom1YHTemOxjHr0plSsPUw5Dv2pZ9T2PXHkUu3sJbh+A07z81pu+VeoffPLi0yf1nv+V+F/58klfgnjISYCdMhvq9N/S6wc3f3lYn//49pmdqwnwKdEsW4bFkN3J+tTjEEjW0LUt1pYkrTAmocx6xGMtRhsIEWsCKUViETHGgdak9YZwjQKlcKVD3Qsspdbhta4cTCmfzKzvBZXNxRfK5H/G5oBTQAr5HymPwEIHUYNNqBAxxmB3tuDsGfo33mJ+0PP6nVv/DPjOib3hQjygTv9fO3EaLfeao8+GWH1tMtkcXLpyhbt3D7k7PSLMOvRWQmtN3+cpxNrm0U40HnPvGdS9qUDAWBRgUsxh0/copbBFQUodvkuYe+td0eegUhpiAmcgqref8164EXNthgFI65J6cqAllUdooQdVQgzQ9KSuJ/kIwwH0DW53k6OD/YNpv/iCNQgh/g2ntvOrOPVevLE4+OU3j/bAObZ3dzi3c45hVRFCIIRA17VorQkxEPpA73t810CzgqYF3wMpT+c5l8MLlT9aB0rTrlpWqxX9qiclDbj1yCnm9bCY8uPLOj8HCo6OYLnMozViHnFFn6cPU8qvee+jivn7bUPyPav5ClYrGBRMU8u/fvEbXwCkfF6IH0BGYOJh9kWzvfW5vfnxc5vlgMnmhIPZJm0INL6n1HnYEkKgA5xVRGNIKaEseRS1niLMQ6T1SCqtA6ZtWc5m+TmqGqdULps3Zj0KMxB8DrFCwWgMzYrm4BgNFOfqPJVYONbzmm+/RlxPP4YuB11KpJjWI0WFDp7X79757kzH/4X2+P17R4V4iEiAnTJntx856Ut439itbTr4wjx1z01vH6K8xpUlS1qCVkSjaZoGVVhcUeA7jy1yKb2L+u1R172pP6XWoyYAxep4zvHxlMlkm6oqYDCG8RiMe8dUocnzGFoBHgZDqp1twv5hbgO1OV4Xa3SAygUfWufwMiZ/XyVIEU3uBKJHY7rFjLfmh/8gP6kQ4geRABMPuy/NK75U+fK5zXJE1VbM9m6w7BugzD0JVaJwBhUUdInSGqw2qBjzFF6M6+k/k0dE2oDvmc1mKKXY3JxANQY0dD7v4UoR+lUuCEkqF294D4MBnH8UY0qa669TqQQMYVDmkVpK4NM61CK4vJbmVx7f9+wf3H3RHmz/5o3Dg98Evn2i76wQDzgJsFNmP/yHt1Vo/2D1hae3zz3XG9ifzjhuF7R9T6gCA1dSkOhiQHnQKaG1wqZIkUKe1UOBKdbPpiAGlgdTvPfs7JxBbYxIqwXt9BjrSuxwCIPhuguHz0UYrYZ2Bn0PwwlUA5RSxNUSPTAQXQ4r0nrKkPxYXQCJBAyGI+DOMyfzLgrx8JEAE6fBl64f7H1kk/KzBwd7n33z1s2rOzs7NKHHOkPE5S4XQDC5Y30kEWLe33W/owbk6b3FjKZpcM4RY2Rx4xbLpqNHESNobaiqIVVVEYKnKBym0LTNgqPDfeoAdVUB0DYt9Vzlfof1II/UIO8J84BfknAs/RKjax67ckl2KwvxQ5IAE6fFt9f/fuWNw9tf337k4rMhJbz39C4Ro7pfNc+683yMEaPTur6iBwLExHKxJCqFdgV7B1OOpofcur3P7Tt30dry+ONPsrW9Q9t2bIyHbIyHdF3L8fE+b16/TpUSH37mKucfu8L0rWsU3uRq+r4F1huhk4G+p+97jNP0bX//LDfjj973N0+Ih5EEmDhV/sW3/xTg1252s2cvDSf0fcIkjUuGMhkKCpSHVeypC3A6rIspIviG4Hv62OdGu7qg2DT0i46VWlFtXcZZy51Zx8IfYYxmtuyYzleU1tCsYGvrIucvn+P8k5fBGMrJNl2/oDqao4YVmIocYoBxuC4AgcIV3Fy8HVwV8OTumCd3P3gi76MQDwMJMHFq/PpX/xVFPQT4jVu3b/3j3SujUa0sfRcINhLRxBjpUKToiUqD6nNBhoYYPMumYxEj9WBMMR6jesVGsmykgvnC4wqD73rmfUvfL6mUZqkSKQR09Jw/f46tRy7jdYUdDKjPROa3bzJdLCj6nmE5zOX33ufCkRABRdSWedud8DsoxMNFAkycRvNF3/6Gh89HY2i9p2k7/m/23jTYsuu67/vts8985/vm13M3utHoASNBAAREgiBIUZRIDSZLcmS5rMSOIjt2KVHlQ2zFVa4M5TiJzFCWXGVZMpVERZkSNdAkRXAQKE4AKYAgCYDoRgPo4b3uN9z37nzPuWfaOx/2bQBJWTIpNdFA6/yqXnX3G849b5/T53/XWv+1tmUrHEciEQghyIuCPJ0ZCQtNnOYkGizXp/Bc4sIix8IOKqiwxsX15+n1ujTrDerVKlJK8kKx0+syHvYBiKVFOD9Pq1EjzHM8IUi0ZBilhAjcJMVxZoYRrQFBmqVkhWI8jq7fipWUvAEpBewG4+Nf/cL1PoXXBRnq1wdx9HPtVh0sSJTCVpqi0Cg0ShVYjsC2AG1ToBhnOeM4IbMkLg6FgCTTbHa2ef7SRZ67eIFht4cE6tUKSwtzeFJy5jvP4PoOSysrjF46x9ZgwNGDB6l4DrWKhysUo0lM23HxC4Vna3zbMXZ6DaNhTIRiPE2u97KVlLyhKAWs5EblyfWtrSf3N1fuyjVMc4UUBVOtkNoYOpQQKF0QRTHac5lkOes7HVLtgD0hLyAvNOtXOrzwwkW2N7cJbAfXlqTjCanr4ddrBNLGsT1UppmmU7Y2t9FY1GcbYroOZPGIKM8Jmi2UTpGBTVFkFFFGrgUZkm63NG+UlHwvlAJ2g+FYlet9Cq8bhln+64nWdwWWpLAEWgi0sMxUeS3QltnEUgmLPC24vL3N2pVtcuGRKuiPJ7TqCyilEVnOglvBtW3qjsPK4iL79uzBsS1OHzjMcDJECdCWppA+SkCUjOn1eviexXjYYxBNaDTmabfq5EAgHSZJilOrYauC3V4pYCUl3wulgN1g/Ob4A9f2gMsrZtzR5UswF0IGP5H/39f2Nb5//Pb2cPC/h7VWNZCSVGuiNMVXEikFWSHJVUFhaeICLm92efbci2Q41GpNwkoDz/ephiF3HD+BleSIoqBiO6wsLrB3aZEiTcl1QX88JFMZqcpJXQfhu0zGVTYur6OVQgqXnd0hm9vbLC4skkwSxtOx2b4l16SZYne3v3G9F6yk5I1EKWAl3zO/f+CXwc1gugGkkBZw6RIcOgmDEawG/MS5D17v0wQYb42Hv31kYfXnJsMJaV5QZBmpI3EdCbhIIVBKszucsL7VYXOnh19r4nuKxlyVRljFtm20snGTAkeDlRcwGLEbRdjCJtc5SmX4oYcrbTr9IbltobIcB4Fte4gKJL2E8SBGCIesSOj1hjTac+hc0B/HdPuTJ6/3gpWUvJEoBazk+8LvL/89iC5B2ofD7/hPfv/Pnvnl78t5dLa3fr3bWP65qgZdFJiWYkWhCrTW2EIwzRWXrmzS2e3jVxs0anO4TkBWFEy6PXSa4OcQ2B6O4+Fq0FlGGkekSmHZFtgWeZGRqALLyuhtdBhNExzPx2k0Udqi7lcpcuhsbSN0wXA4JNWwVKlzaW2NjY2NUsBKSr4HSgEreV3w7479Y6jWeM9n/s61PvSTO/N7aCysYumUtFDoIke5ZkdmYUniTDGNM4SwabdbVPwKeRTx4pnnqDk2y3OLYLsM7RQx3UEkGbIo0FlK4LlkSoGjcGtVas0mjrBwF+ZxqjW04xFnOb3BgCDwCYMqk0mMLjJypZkmOVE05YUXz9OYX/zrJWBnu9f7DEre4JQCVnKj475w4QVWW/Ng26hkSqE1pAUTnVIEFXJlBmNYAqTKmWs2qM7Pk8y3EUVOq1pjLqhQlx6OtvBSjcwVRRIhhE2lWcWpBGjHQtuCWEUoCgoB4yzFzQXCDhmOI3KRMcXY8zPLRzoez65f5syVy7T2H37iei/Wa8pXzlzvMyh5g1MKWMnrik+96V/wd9b+12t5yHpvbYtnXzrHwb2HqHsBJCl6moDlECcZQmmEEKTTCEdr9rVreLaDu9ggT1IE0HYDqtqm4vg0giqOds3WKkKA54INsUqIiwRH+zieJtMZrrBJdIGMFONsyMZuDxVWsWyXWEkkHmc3r3BxONlowXdt4vjggb8HlmO2cqnHMO1yp+5fy3V7DfjU9T6Bkjc4pYCVvO748OgH+YWj12wrrHbVqvPS5U1cr0EXh0BY6GTC8rxFIRMatTrjaMpkMub4kWOEgYcvJYFtIzwXnefYCKI8Jc00ypH4UpGTk6YZurAoUCRFhmULXCfDygRQIH0HWwgKIRjFKWtXtpjKGo2FFYKgyfbaBme/cYaqVXnyhecu/oW/yCf+xj8FewFGAtQbTaxKSq49pYCVvC754PppfmH/NUkxHV5Y2cM3H3+Kutek7lZpN1ukqabYHVGreKDGrF1Yo9FosbK0hCclUmukKvAcG0tIojQh05pcpWztDolHMZNpTDSKKFRBpRbSqFapVAPaHsw1qiAFBSCEJEcQ54p+kpFsd9meSOrNhO6ldYb9PifvueM/Wv/6rbn72bQOQlADyppRScmrKQWs5HXLJ0ZvZ++FX/mrHubQ+x9+H54f8NK5c9x56k7StGCzO0a3BGkSszbZIFGag3v2EacZYCEp0HkOKJTWpOmUSOWM05StnS4b2zsMRmNUnlMkGftWl9nrrOBUJJYSWEKTa01eFEyFRZxb7MYZa50B/jRA2zn5S5cZdy8T1Cvkrv2ygP0fl5fhyHFYPcxyp9yUuaTkz6MUsJLXNV/Y999wxzP/01/lEHfoQvDwgw/zyEc/xtlvPclNN59mfn6OLC/Y2dym39ul7jn0OgNWW/OMxxOEZyPQZCiEVjiOjU5TxqMh3VGf3fEuu+MJC802li0QjkQLje86uMFsI8xpROqFTG1NbzxhNMkZp4LO7oA0HeOGVTZjRbPiEGT2E797MYP99wJ/cSqxpKTEUApYyeuep37gX1P76j/7S/3s7TX37YNhzIkDRxneeQePfvrz1CtVxM4OQbVFtztACoft/gSkzdrGNp63ikBhV3wm6RQpNK7vU7NC4nrOPjcgKRSTKMF1fZqtkMW5RZYWF6hVq4S+i+1ILOmQ5orOKGarH7HVHZEUUGhIC000BbX3LdRPnyRfnftXXPz8PwA2r+3qlZTcuJQCVnIjc1dkz980SVy0ktz/5rcQb2/ylSeeYc/RmximOeNpjshSJqMB4zjCtSULy0toS+AUIG0Xz7ZRUuA5DkteSFtDs9Xm0L7DVGsNXAE116PdrLHQmsPOM9IkRjg2w3jExa0d1jq7DApFYdlMhlPSQrBn7yn8u3+cTm2OLw3HP8H9P/121l78ReDD8KoNpEtKSv6jlAJW8oZg9GMfgUkHzn8LvvkEjLdhfxWSmfN8dwD7j8PBI9BswXYHJtu/uHz0OJVmHWXnCDflxKnbuLi1xbmXzuPOrdKPUqwsx6YgLVJGyuLc5hZ75tuIwKfiOhRSIl2bSsWnXWlQFJqlQtNvj8iyhEpQwfM9sjRhs9vFlw5JljHIMrbGMZujiO3emJ3ugGgSkWcgcrjnrjt4trbCUyML/CpM0xaHln+TQ7f+TXbP/Rxw/roueknJ65xSwEpuVP6L1lt/4m92pzlrRcxBX9O2BXOrQ07cdg9fu/hJst1dsDxUVlCRAp1ptgZDuqMBkyyhcBzm5+rUbR+tFGk0IS402SShXmkiCsjilN40xfUD4ixinEzRSU6WKza6PXppxvZgxFqnw+bmNo1aG1GktOdaPHDvnZw5N4UoBlWDSh06MbiVd9I4+TTEvwR8CFDXezFLSl6PlAJWciPy89z/nl/rvXiZx86vs1WV3HHHQWJtM0kVwg04fPRmnnrhApWaR1pECCDPU85f3qLZqMBGhyjPWRnNs7C8QGBNcYuEdq2NyBSeV0NlBb2dPlboUgsCJlqz0e3h4bHb7XN+Y4teErMziRgOJqRZxnA0gGnGO977Ixw7vIf4yS+DkODsgakFBKAC2I0rTPx/uend+ZPk3b8LlHbEkpL/H6WAldxoPETz6Ic4dwUuXIJRH3nlMs5xH9yYsO5x4Mg+blMFl7d3iDOFpQu0luRaMhmnKFWQJjm9bp+1zQ4rOzsEQrBnbh7LEoi0wLUGeEKAY9PvjemOY3JHMIwyKlKy3Ruw3tmhG03ZjRJGcYzreowHPe47fSvvesudrFY0B/IeXNqFwz6kCbjzkCooFIwLSO17aR34BnT/Z+CfA+n1XuCSktcLpYCV3EjchL/nY8SuzaVLcOEi9K6Qd88S/uARKq6NdDW64rHcCFhtNXj64joSi9CvApCnKXGkcCxNlqUM4g7DyYSGVyMaW2RTyULo4kmXmu+TakjynEIpJD5FDmcvXmJnt8tgHJMqGyEDhFQk8ZCm6/LQPXdxYKmJHw9YSCYsXl5nu7YMdga44AK2C5mGOIWscAndf0Zt9f2Q/V3g69dzkUtKXi+UAlZyo9Bgz+lP4S00Wb8Ca+swjKj3BwTThAW/iptPIC9QWnGwPcdD991DYUlefPE8o2gXR7gIYSORZKrAdiR5okizCcFiwGC8w7m8zyAIGU9a1EKXubk22rVRSjGIhly5sslokrIzmDAYTEmASCnIUgIhePNtt3L86BEsneH6LiutkGnnMizvh2YNbGnmKwoLLBtsAUJDUsDZndPUw8douB8CfgmYXOc1Lym5rpQCVnIjILn/vR9j/vhROhmsX4IXXgBSFtAcmJtHpjmeraj6IRWRYdkJUavOodUlRru7TEYRBTaZLkgUMJliZy6ZzpGuzVa/y3CsaVV8ullGp1tn/8oquWVh2z6jacRWt8vG7i5F5tDtR0TTglxAnia4luKWo4d478MPc2RlET9LoJiytxXgR12GG2tgtSBcgMCHXECBicRyBZMc6ksQ5xaT5BcIwh+llf0c8Nnru/QlJdePUsBK3tgUR+BQ+0McuPsdxA0YXYDhDvS28YTCCwscIXClg9IR8XQMSlH1bBZEyKkjB8nGYy5duERnEJFrQWB75CpHKcgKjRYwlSlaK7zCIxsOieOUWm0OJ0zJ0oiN7W063S7jSUxRuAynOUJIsmlEIC3uPHmc++++jYMLbbw8oxb6kEbsnQs52LIZ71whqqyAPw/CBTyQPggbHAuwjdkjnwICOsNDjLNH2Ot+GPhFoHcdr0JJyXWhFLCSNzI28EEOvOXvM23AqIBJDBfOQdyhHYSE2PT6fTrjAS0vR2iN7zkErktNppy+6RB1z+Pc3BzfevZ5Lmxso/OERGeoVJCpgkIpHATZNMEubPJIoJyC4STF6ozZ2tlhY2OLtMjN9I1kSpoVCAqKYsqhPQd40+kTHF1ZpuU6hJZGUMB0TM2H+ZqFt7VBWtkktxrgVSEUYHtQZKBdcDyQCqQNV7oQupA7gjM7P8vtcz8E3X8A/P71viAlJa8lpYCVvFFpseeBf8/KyXdS3QODMUx3IOrgTK5weClkOhgTTy28quT5tSvcd9cxklGClBa2EMgsx8pilpoV2L8Hq1A0qhU2twcMJjGxKggch0wXRPEU37YYDVKyLEHbkrX1Lh05YTwZM41zpG0zmUzoZWNabgUHuO/W23jgnrtYnW9SkeALhYMywiTAcSQtT7LHYdp2DgAAIABJREFUFZxfe57AqTGqhMDKrBYmzL5fQkAyhp0ueI6JzKQHexZgY3OZivcxKlSA6Dpfl5KS14xSwEreiBzl+IOf4NjbjpE1ILJhOoX+Dmy8wB1Nwen9yzz29W/jO1XiacLXvvE0x04cwHNDLFLGk4hGJcCKYshgrh4i9++jVW+y0exw/vImvVFEb9InVRlV6SOVAAWe8Emzgq2tbXzLxbYssjwhSVMKNMfml9i/b4XFdpvD+1c4vGeBhivxpEbkUywhwbEhz5G+hycld9+0H+vZTTZeepZWxeOSL8GywHfBbYHS0OnANIXVJsaq6Birfa0NOkImnVXghet8bUpKXjNKASt5o/EwP/TTH2VxX4usYuIN7cI0g84W9NY5VE25+/AyLz7xLYajEaLq8dzZFzn30mVuPXGQaJIROCFpkmKj8KXAClxsBJ7tUKtUqAQeL754gYCcpEjJlCItNJochcS2LBwEkOJbkmbNoz2/yP59e6g2KrTrFVrVGouNKjWpCS1F6DlIS5AXBU5RQFHghQ3SKGG15fHuO27m3z35Reo7Ldp1n25QgWkFkj4UNoRzsBxCowk40BnAMILQgbBBbxgtUApYyV8jSgEreSPx85x614fwqjYUMNUQBhBpGA5g0GEl61Mb7nAodDi9d5HHn7+InfskheSLj36Fm4/spx7UYTpFFApXJNieQypBILCxcAB7dZk8jtm3vIBGsTsekqBQmUbkmjAMqYYVVJHQbFZpNepUQocgDKi4EmnZ1AOHqmtRtRVVTxJ4Fp7nkqocmbsIV5AJh3qjRX/9Mj/+g+/l4pkzPLv1Ar5vgxVCrQp+A5rzcOQwqMykEV0PKm0oLGO1T1NeWLu0cr0vUEnJa0kpYCWvB767yetzJ2CUAQJkYe7eIoMsBjEFqQhHY+JsGz/LePMtR3jpxct0RyMWWg0unlvj0x//DD/2ww/jCQfXykAJHMcGrcEFz3YhUwSOi3/zEeJJxHgaEVRd8iKj0BaO5VCtVAh9DwuFJRTNRkglcLGloFqpIouCwHeoexaeVHiORdX1QVpIS2PZFhmQaUWt1mbMhJCCB+86zoUvfYmtyxdh8QgstaCyAvV9MzOHC1UBWQq+A0UORR9UCkutxe/nRSopeb1RCljJ95+tSzDcgrX6n/89B26DqgfuATiyB/IxL2gFlQqIKiRNcByoOZAD2oc8g1EXdteAAdhwIYVFXXD2pWe579bTfKc25EI/ZTJxUMESn3r0O4wTm//6H/0MyeZ53NwmTjJQGksoQsdG1FySrKASzDP0xizkDXYHAZNkymQ4IplE5GmCCnyqtQDfsWk7NiIrkJlCJhMarRq+65FLjRM6BL7E84AsMU5CqbDcAiuJmA4t1i9rtrfG3P/m43z2K48yzBLalQZnmw3IHIgVjPowV4V6COMURApuBFkH7CHHp/nya3RFrwlnrvcJlLzhKQWs5LXj/iPwzOOwdRbUff/fr8WA6wMBODm4NUimkFpGwFIbphjvQqohSo2AKQVWDvEQogkFAduqyfNnLvPuW0/yt9/zNn7j9z/JU9MNpuynXlng60+c4cO//ju87133EfgtsihCqRRHFqgipx74jPIJ0ySmYgmkHyK1Jk4DUtenUBlSa7RQ2AIqUuJrgbQsAsdnPqzjhRVUKMkchZaQ5SkkwpgxQh+lBUr6PPaVr7C93sG3QtLJBFu5LNQ8Xhhk1LXg7Jkz4ESw6kJNwmgIieReobmlGNFyJuROxiiZ0E+nS9fqUv3Bj/1TaDowGZodOPspDDvQH0DoQXrpWr1USclfmlLASq4Pi5uQu9BvmX8LDdEYMgWWAompb1mOeXjqCNLpzEJuQZoaMRAC0EbsplOqVhVbHeTF9Q3OP3uBt779Nu67eI6Nb1ziXNLDkT5a23z2c39Ksr3Fe9/zdg7u3cfuzhWE0Hg26EIR+uDLlCLJ0ZnCCXwiR5K7FgCqSEinU2xHErjGnGHbLtV6hWa1ibYFGRkSTcV18SwLbdkIyydVDoXd5Pxmnz/65OeI+zYH/RYVEkgiirzAEzbjjSvcfvdhvnllCzqAqPEzgcPDGRzRKd3tK2xP+qhmwVrvJVpB/D0L2C+f+MdQ9cGrm2h3MoY0x4S5JSWvb0oBK7m+LFZgqCGegoggkOC64IdmIoWyIAhgHIOjjei5PigBUQTToZnirgtEHEMW4zrLXM52+fI3zrLsTvmxO++lvxETbKV8bXKZQlbYP7ePP3v6LMN+wsM/9BBHDu0jVRGWBVYxJQgchJQoEZHbGqsQiKkgExJpCYSwUYGP6zo4loXlSTzXoVarYUsL27dxbQtFhi8lruOQ5mBVqoyESz+Ff/ORP2Ttypi91LGnO7TtRdQ0QjoWWidEaxcRk4x3HT2B1II0GXJ3ptjTvUzbz9l/cIl0aQ+1Y/v4xKd2+OJz3/gLU4i/dfc/MevqNWASQN7AKGNJyRuTUsBKrif7gV8hKqDlQqU6Ey1gFEE7AOkaq3iWgD/rn0KZtFauTApRKcgyjk9ipsQIZTNA8nRvQvgnT/IL717iP3/n+3A//RkGyTrnRcrF3U32hQc5t77LuV//CA8+eB9vf/tbcEKfTGuyIkYWCaFrIVAEtsR1JEq5oDUaDWjyNMeS4FgC33WwBGhb4DsSy3NAOCAtojihvriPfiFInSp/8PFP8+XHnyMUAU4eMSdhfytgfXuDIs2oWDYtF1bqgmce/SPe/ePvQ1sL+Iw4+o4D7P+BE7Bvidir8Nx2j9/7SIdBpb4A8NWFw9CoQvVWCPeAlpC2IC7TfiU3FqWAlVwPbOC/5cS9/wMLt1Q5exnWJ1Ak0PTBts1HXhiHoaUgjsDyIfeAwgy6VRq0gmRKK024o1Xl5vmTPL9+hnPDmH4uWC+qfOGxF3jw3oC/9a4Hyf/0j3m80+NMN4F0RNWro5Xi049+kfMXL/C2t9/H8aMHaVc8VGxhOQIRD5GFwi00QgiKoiBNU4SwqIQB0hI4roPv+7iOh29rlMgpkhy/EoLtoPFZ7w4J5vfyx48+xu997LMUmaRiQVtknDq0yN65Bo8/9i2SRJEXQ455mpV8jGVHnPujj3LbD3+AB/7h+3Hfsswj0w0e7a7xua2YJ1/oQuHDkbtXyeYhPnudL29JyWuDvN4nUHKNOfkj1/Z41RroAkYD0zCrgPqKmcuXjzFiomEwgNYiJKlxCqYZZAMopuDOQTKBxgpsrz/A7W/9OKfe8tPM3+IimmaGYXdixiN5vkkh2rNIK08gm4IWxjKeKdCWKdEkUxAZDDY53t/gdL/LDx9s8ZbDLs7WkCJxGBPQmaRsbJzn1lv2cvvpY/i9Lh6SKEoZpROmxZjA9ugN+zz1rW+RFgkr+/ZSbdSJkik5ChtB4NhIKRECfN/DcRxc1yF0XVzbwpEWtiWRMgcUwpLYToVYSVSljtNc5pEvfZ3f+ch/IE8lbTugPplwqiZ45503I6XF186tca47QAqH21ornGrWqMuU7d4WuZzjwt46PzK4zP+zfoGvrPXZGPswCmHpKMimw2S0RL77CL6rcJfAqQMWFAHkA7AdsH3jbFS+MYi4tpm76LrGnl8oCJWJeLPENDlMC0gimCYmCi4Gf/V764sf/6sfo+SvNaWA3Wi8fgVsnsbKhzj94Ic4cscSqgabKawPIM6gEOY4vjd7YW16s/LMGDZsZ/Z9ykxl15Z57XwESY9TvU0eCgU/etfN7Il3uC9cZHOtwwaa53TCyM4ZXXyJ017I4bc8SGU4RuUpVZXj5AlSpziWJFeaZ146y85WFz+osLq6B7BRaYpjCbAsCg1CyplxQ2BbAgFYAqQEyzN7eFXCOnEmEZUWEQEf/+yX+Y3f/AhECj8rCCYRt1Ql77hlmZN3nuA73zzDN6/EXIljXD3ldrfFXidkMugTZYrndhMu7lvgpQKo7oVNF/pN6LqQVSFYAtG6m6D2AMX2J3CX4lLASm5kSgG70Xj9CZjAnftZjr7tj9hz9wPQEqyPYa1nxkCNphBWwbOhNzS7ENvWLD3IzGU4EzchjNAxG3BrCxh0IB9wYusi/+Udx5hLIuLf+Tie1eJ4bQlLBaxlQ3p5hkwtpttjFlLF4fvexLGFOv60jxyPcFSGKgqU1tSDNhsbHb7zredIk4LVpb3MNaukaUKSJmhLILSaCZfAQmOhcRBIoZG+hXBsFD5ufYGxVeVTf/p1/vCPv0CegDMtaBVwS6PKbfM273rLLajeDo8/fZk/206Zas0CKe+7+SSnVw+zubPDd4ZbXNYZXavCVmUfdHyIWjAKQIcwzMCuQrAAOjhEffX95JPP4dQ7pYCV3KiUAnaj8foSsFPsv+tjzJ/8h7ROhIwD6CnYncAghkSZgbW1ipkqEUUQJ2AH4Pvmwam0GZuUJuZ7hWWciUKCpUFFMOnwtnzCBw4us/3hP2BON6Bw8XzBvpZPkECWWlzMMzZTycagh9zd4fDeOW46tMqB0CObTLEtD5TNMM0J3QYClxfOXaDb6TG/0GBxsYUlHabJFNvxjI1eCqQQWJhIzLEthCsQjoNXaZJZFT7zpW/wWx/9JN1xRj7NWJI2hwKfE60q77//FNa8zbcffZSnr+SczxpIy+JErcLN0qEhqqhana9tnGeLiKhrcXTpNtYGDWgfBLtirklvBEpC4YA9D323TXXlZ7DG3wbrXClgJTcipYDdaLw+BKxCmv2P7Dn9Yfy9h2jeBAMHRpaZIDEYgyogTyH0Qc62DdEaoqnpQ8o0VKvgBRDHIB3zYM01WNLUxCQQDaAY8oGmzdzZMxzTHsQ1yGOwIrxhj+N7D9JUVS7EKRt2wMZ0TDEYUqxfZFFntG+/lVsP7mfU3UVlRmTyQpEXilY4x3anx7PPPI1lW6we2IeyII6HBJ5Eao0DeNLCkRLHsbEDGyeso905HvnCt/jQv/l9ChHgCcmCVLTSCbevzvFDbz5J7eZDxI/9Kd/ZGvDUjmYolpi3Jfcst1lNNTsXdhGNJrJVpxt1iGPNnH+IK42DpHZoxKdVh92ecTwOYzP0V7ThysBD2D+Fn0YUwVdLASu50SgF7Ebj+gvYe1m5+xPM3/LDsCQJ9kLkmokaoyH0OmZqRhaDhenpyoV5QFquKSSNJiBysxOxyk3vUoEpMInCiJ3CfK1IwMp4cHeDU71dFgZ9yArjTtTamEKKgtXlOWpJShIPGCvFC5ngytijs1vgZSnzN61w7MQKC70L1KZjgjSnYoeM0pSpKkhzl68+/U0c12b/sVVsv0DnY3wlqEqXih0ihcRzPexmm1TX+OLTO/zzX/0U2EvMFy6H04jjxS4P7A+59/g8q/fcAV97nj872+PzA48L9iILqsqbioA3e1WaSjIex6i0oF3zkH7GpV6HxGoQ3HyETceFRh2SDI4dgsvbsDgPu0Oo16Fah/WuRey/i6p1mHzwx9hOUQpYyY1CKWA3GtdPwGxaix9i9dZ/iWw2SW0zRd32YKJgNILeAMYDKFIjTmEIjg+eZ3qVhDDTN0Ibul1j3qj4xk7vVqBRmX0v5oGaFWDlhMmQu9bPcyoasphmJsWoLROl5RgjiFAsVUNECpM0RwuPCbBdpAzShLizxYprs/S2t3JyaR4rHhFHXaQFSudk2qPRPMDTZ85xpbfL4WMnaLeXUcrB9WsoN8Cq1EltBylcnnj6Bf6X/+03ULJOS1vsYcoxe8ztCxZ37J9jzzsfhDPP8/xjz/ONXs6zU4ntNFiIMh6eW+aAsFDjmKzIEYVNPJ5QW6oSVpbZzRyS2jxrdgC1lumHq9ZgtQHrHTPVJJ68EsH2xzDJbqM19xAi+iS2PykFrORGoBSwG43rI2AtbvmBP6R9/KfIPCgk+FVwA7PhYn9kJm1EkRETKcBzzQPWssCyIS0gz83DtEhNtFYUIC2TMrQcI26ubYb6BhUTfZGghzvcvv4Sd+qUpSKH3DapRqVMJCYl9MdIbbG6uEigJdN4SCxyNuyEflYQ5zajSYHb7dM8dZz9h5doFWMmg01cFJly0MIjFy4XL+1yZWvA6VvvoTG3RKIVbq1B6vmISotnz5znV//Vh3HdJk0paCQ9jjgRt80J7tjXYOGhB2G3zzOf/yrPDjXPRZrE8jnotzhZeNzTahEWKWI6NqZLbZMkCVEW017aR0KVkVXhrF0BJ4SFJRhOoFUxaURymE5gMoF2G/zAXINxvA/sn6Rif4HM2SwFrOSNTilgNxqvvYAdZfHU5xlX30zaBOGZnwl8GOfQG5tIKZoagUIb96CURrgKbb6eZiZykBqikRGwLDW9XrWKGe7rSlMfyxUgTa+YlTE37fGmnQ1u11MWkxSUax66eQpq+krDMxYyU+zxQ1qJTV9FXHEVkfDZncDmzgRpSeTmReYP72H+9pMcIGUy2KHieez0+6hMsdw+zMb6gMcff5Kjtxzm5K0nyXRGvd7ic3/yGB/85f+LKLWZrzegv8upeYdjlZRblwMWH7wfCuh9+SnO7aR8vpez61aYt6rsGSjes7KPZpZBMsYuCuxCYmkb23LJsoidzoRIeYxFgFVps4ENC4tG1HNgJTDRp8hNxFsA9RYEdRhnkMgGE/4Wof08yv9OKWAlb2RKAbvReG0F7B3UD3+GONwLc9BqmxSfKyHWECXGjBFNjRDlOej8lYapTAECktyk+wIX0NDvQW8Xslm0VhTQmB3bd0xEIR1zfmlMczrgtt0NbknGrGhl3Hjy6sipfGbHt8z8xDgB26U9v8BC4NNNpsRTTW4FFK7P9u6A8XCM3emwXKsTnj7JiXaTJOpQlQVu7tEbpDSCNlDwra9/mclkm9X2PI984hE+9tuP4IX7CbwFZFawt26zPyi449A8Bx68F7yAi5/8Ei/1FE9uJZxrzmM7dQ4kDm9SITdX6zAYmvXSGlsJM4dRQ6ELhBPQiQvO9yKYW+ClsAq1uvlIU6i6mOKiNms6TiCzoF2FqQW4MM5dJnyAagBO9MVSwEreqJQCdqPx2gnYzyPmf5vUryCbELRNRORg3vVPZjWqLINJZP4schDMzBgCstwIUZabaCz0IIlh2IPdLrgWVAMYTwEHfBdsaSKwZGbSiMeMetvcsn6Bk0XGfqWMUArLPIxVAcjZM70wv1OaQ5TQ9AMO+HMQJYyKCOXYjHOFZTcYDnJGW132Bj7W4b0cPHaALBpgBfMoXWM8ybGkJM+mvPT8Wb7xZ9/m209dRNEky+qEbp35hs+RuSp3HdvHLQ+/Fap1tr/6FM9sTfnmVka3usS2H9AYK44OC949v4Kc5jCdArmJTrXE1gAahSJVmtR12RUWO1ryUqUOtYYxbEzGZgaiFrNhyB70IyM+2jU1xDg11wJbMJw8iGOdoGZ9CtvLSgEreaNRzkIs+V6xgf8TvfT3KWzwKuCGRpxyz3w1w9Sg8pmAaWV2TmZWj5K2iaxsYfq5mFnjk9lU+jQzUZcdGNu3KGBn26QYlxYABzLbPOiHMRQWw9xiKGwTgeghCAUp5rhoMyRYp0BhxK1Q0FOs1lv85IJgdbrFE8mIS8JjJ7KJCovdccZG9CynNrc4/eBt3POeH2fr00+Rr/eptRpsj8cEfgvbq5IWEuFZOKKBjhwCSyAmKeFChcbCMkSCpx7/Che3xjzTSbkQubi1BuF0wuq44E1BE0dYRsC1NkYUHIziQyCgISRjcpqioJVP8Mcd9g52WB/2YLps1jbV4AvTJO4F0GjCVh+2t0EuQiOEfDp7Q1HAjv4AWDdxiPcB66/97VRS8penFLCS74UWR+/792TNdzLUEDZAzsRLK1AJxC5kwohXnpto56qlnZlgSXvWlIyJFmzH2Ol1DlFmRkYJC8KK+ZqVmtTh7pZ5jcYCRI5JTfoBHLmJpaxL/8zTjLOEqsCInS1MOlGlxgyiLEAZUVOFSdN1dhFtl7e2F6n1Cr4yjOl4IbHjMiTlma1thuzw6W/8DpEl6MYeKlwhmk5Y3dMiGncJ/ApRoggCF8upsFhRBPkEOxmwsd7hM1vnGQy6yLDBmJC0sYwWinSacTyHe2yPU0uL0ItnrQHa1LEUgGWGGQtJVbg0iWnamnYSU5sOWBr1WB9HJspdXjb9YAfbEBVmaslcEyap6c/r78JCG+ZqRtCSHIIqdOI7sCd/xvHKTwCPXcf7q6Tke8K63idQ8obhKKt3Po6z8k7GEpwWuHWY5uZBWakZYYiS2WaTaiZiV1OH4pXNJwtlhC3JTZpR2saVyFX7O+AEJoJQs7FSnR0gNZteJglUHFhehPk22D55c44oqDIWtkkVamVez5GAnKXNBODOtmEx8wohgcEI+oo76vv4keYKe+IxTtYnkQUTr8pW1iJmL5NxDQubdHCZOXeX9NITtLNtlvI+1XibltrBm7zInLvGfLjBXHVAPLzMeDJEhi2soI3tNti8vMt8JeCAo7kfm4fay8aFOR6ZlRaWiRhxzbmrWU1LQQVBI1fMiYJWFlOfTHCGQxhE5s3B5W0Y5VCVJuq1MFGXjXEmdjpmU9BmHUIXpiloB/r5Ms9eeRT426/1jVVS8peljMBKvhse5t4f/SjUWqyNgRCCmb0dYZqFwYyHimeDd9HmXX8xSyFacDUdZgRkNuuQmY2+wIhZoQHHbGJpexDNUmrdHaBu6mz9HtQC8OSsFyylqDfJwxpba1ssO5i6mtKvHD8vjHlEiNnrKrBTkIVp6u3lkNgcbNV5YH6KKgacyyPs6iKxCmnKKu1miBPGCNFlaV4iIp9m4BNNpoQ3tSh8h914CDpirlEnHlpEc4tAlXHiU9gt4m7M3lodazLisONyl1cx0ejOwESFQhhXYG7N5j4WxpkpgcwmUJpQK5qWplUU7PdcjsUpz0aJiXy9ELoRzNfNTMnp1NTFxmNIhKlxdQdm77WVKmx3zHrKCkjX46X+b7G3egr4782Ll5S8fikFrOQ/xc9z8/0fYlqz6U2B0AiWtE29RkrTlDyYwFZn5iasmM8VVwVpFugLbbZMQZi6ljPb90sKEyFN41nTMeB4JqLIZ/MSQxeePQuHDsCSMBGKK2bilDJ0HEa1BtteCOSgYhPp2ZZxTGKb9BxiZkLIgQKyMagQ7AZMM4gKTiy1SXoTRuMx0xrs5oojtRo/9UNvp3oyhD05OFNIJqgvPI5lV+GHfxBEDBeeZuPcd1h56w+C7UJegWkD/WyPf/0bn6TfnTDvV9hPwT2OR4UQRomJKi1MRGR7s/ShwPxltoZCIIWkrnPahU0di1BonN4Qwh4cmEC9YVKrsm4GJPf7UPehVTPzJKUDG11YlLDUNtGe55nrpKSpKX79zH/HQydPgPrPgOFrfL+VlHzXlC7EG41r60I8yC0/8Fn0gkV35vwL/FnfkDCpwkYFen3Y6UA6i5Yc20Q/+czCnmOEzbKNKAnzMMaWRpxsadJbo9mUjiKD5QWTVpvM0pGToeltGvQgnRqjQmCBr0FntFVOy7HZXbvMEZlTz6UZUWVlYKvZ4F+MJlizmpyWs1QdYCVGEBXQT1mpzLNXeHQGQ8ZeSjrsEu1c5NipKkKeh+xFWAgRUsOtJ2DtKb79mV9h6b6D1NQI9tUhegGm27Dd5/E//jpnX5wwIWS/FfBWXA74NRO1Xk2jWtI0IqvZ6otiJvra/FsCjsSXPllusWEFPO8E7MgKe5f2cSWow+KccQrmNoQS4ty8Saj4xs2ZzuqLw8S8lhcYoY9Ss75hYNK14+kxlhd/FCt6BE2vdCGWvB4pI7AbjaV91/Jo7+DS9swM1zAPWFsaQUlTM0ljHMPuAIZ986ANa+YnJbzcjyTULH1n8XIaEQHSMwKmZ2m9YiYgvm/SkDo30V48m2kYVk2Esrsz+/4MDh0C2yHXAlWrops1BoMhe8TMz19gSklXReHl159FNdIzacQiNRtn4prfc5BzYGmVBywHEffYDSXf7PW48G9/l3/0Sz8D7b3Q8OlPnqByoYNz8Cht4dP9D5+jk+5y86k7YfEQjD2+8/E/4YlvXiIo9nIcl1OFZH8YGoF+NYpXbSPDrG44O1X0K5NJbIu2G9DSNmIc4dhTRDwx/WNq3qxfPDXGl3oNxhOo1WDvMpy/bNZ7EsPuLuxZhFoIeQT9CVQrsPcwXDgHS90T3Lrn6xTr7wcevZY3VknJtaA0cdxwuNfy4yGGkTFqZMVsg8nCPEiv1pMmE/OwjHNTgxEzkbsqFFd3erRm0dbVLVGsmbmCWf1LW7PmZNvY8oVjPm/NzqXWhCA0vWBCm0hs7QpcWoNsykho+sKisneVoZrtHXb19r66hxhiJpazj5ddkbO+NKWNASQvTDrxSp+bGwu8O5ijNc4Iwxbbl20+/ptf4tmPPQFXpjT37ePSi4+C1Ow98U6GayHRGOhn8FLExQ8/whNfP4/nNWklOXdMFG/2GqBt6E1edU7MPvSrruXV9ZpN32f2BkBbtITNnBIcqIbU8gw1GdLOpiYKroazNxk5VCyTno1jqGFciZ4DVcfUw7Y3oBVC4Bizx2YPwiY0VuHiEMZum27wCPDz1+4eLSm5NpQR2I3Gxsa1O9bcnoewZykmezZbMCtmNSofhgMzg288NdGELXn5IVtgRMG6GoXNbjXBbDdlAGk+r3KTzpO+scyHAS+Lm1YgA9PDpWczET3HiKKt4dJlKDTqyD5Szyer1xmJV9/Wkle8CFeFTJvP68L8bnpmHLFmKc+rzc8Z0I1YlS4PyBqfv9Bjfvkoz31zh83dPifvB+YXOHLve2A05Ct/8FHuf/hn2eNegbQCA4/L354wHTcpJg7LmeAuPzQGjdEAKp6ZRqJn6c2X616zPy3rlSS/YiZi2vTYYbNQFOxzPM6kBTuDPjKfmOjUn0WRcQoN2wxNLpTpDWtXZuaaVzWZX</t>
         </is>
       </c>
     </row>

</xml_diff>